<commit_message>
Split releases into per-product tabs — 17 sheets total
Replaced single Release History sheet with 7 per-product tabs:
  Rel-AG ONE, Rel-OneWork, Rel-Learn, Rel-Safe,
  Rel-OneHire, Rel-Spot, Rel-Pulse

Each product tab has:
- Stats banner: released count, hotfixes, planned, latest, next
- RELEASED section with colour-coded release history
- UPCOMING section with planned roadmap
- 5 blank rows for future entries
- Product-coloured tab and headers

Sheets: Team Overview, Resource Allocation, Project Roadmap,
Sprint Tracker, Member Performance, 2026 Targets, External Projects,
Release Dashboard, Rel-AG ONE, Rel-OneWork, Rel-Learn, Rel-Safe,
Rel-OneHire, Rel-Spot, Rel-Pulse, Release Standard, How To Use

Co-authored-by: zainabbastahirag <zainabbastahirag@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AG_ONE_Team_Tracker_2026.xlsx
+++ b/AG_ONE_Team_Tracker_2026.xlsx
@@ -15,9 +15,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Targets" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External Projects" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Dashboard" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release History" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Standard" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How To Use" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rel-AG ONE" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rel-OneWork" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rel-Learn" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rel-Safe" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rel-OneHire" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rel-Spot" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rel-Pulse" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Standard" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How To Use" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,7 +33,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="29">
+  <fonts count="31">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -164,6 +170,18 @@
       <b val="1"/>
       <color rgb="006B7280"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="00374151"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="000369A1"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Aptos"/>
@@ -394,7 +412,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -569,22 +587,49 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -616,7 +661,7 @@
     <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -628,12 +673,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="16" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1351,6 +1396,2245 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="003B82F6"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>OneWork — Release History &amp; Roadmap 2026</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>All releases for OneWork  •  Lead: Abdullah  •  Team: Abdullah, Nastaran, Jawad, Geena</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="22" t="inlineStr">
+        <is>
+          <t>Released: 1  •  Hotfixes: 0  •  Planned: 3  •  Latest: v1.0.0  •  Next: v1.1.0 (Jun 2026)</t>
+        </is>
+      </c>
+      <c r="B3" s="66" t="n"/>
+      <c r="C3" s="66" t="n"/>
+      <c r="D3" s="66" t="n"/>
+      <c r="E3" s="66" t="n"/>
+      <c r="F3" s="66" t="n"/>
+      <c r="G3" s="66" t="n"/>
+      <c r="H3" s="66" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="67" t="inlineStr">
+        <is>
+          <t>✅  RELEASED</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Release Name</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Highlights / What's Included</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="69" t="inlineStr">
+        <is>
+          <t>v1.0.0</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>OneWork MVP</t>
+        </is>
+      </c>
+      <c r="D6" s="70" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>29 Mar 2026</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
+      </c>
+      <c r="G6" s="70" t="inlineStr">
+        <is>
+          <t>✅ Released</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>Employee mgmt, workflows, task mgmt, dashboards, reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="73" t="inlineStr">
+        <is>
+          <t>📋  UPCOMING / PLANNED</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="n"/>
+      <c r="C8" s="60" t="n"/>
+      <c r="D8" s="60" t="n"/>
+      <c r="E8" s="60" t="n"/>
+      <c r="F8" s="60" t="n"/>
+      <c r="G8" s="60" t="n"/>
+      <c r="H8" s="60" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="74" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B9" s="74" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C9" s="74" t="inlineStr">
+        <is>
+          <t>Release Name</t>
+        </is>
+      </c>
+      <c r="D9" s="74" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E9" s="74" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F9" s="74" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="G9" s="74" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H9" s="74" t="inlineStr">
+        <is>
+          <t>Highlights / What's Included</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="69" t="inlineStr">
+        <is>
+          <t>v1.1.0</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>OneWork Q2 Enhancement</t>
+        </is>
+      </c>
+      <c r="D10" s="75" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Sprint 11–12</t>
+        </is>
+      </c>
+      <c r="G10" s="76" t="inlineStr">
+        <is>
+          <t>📋 Planned</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>Advanced workflow templates, email notifications, calendar integration</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="71" t="inlineStr">
+        <is>
+          <t>v1.2.0</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>OneWork Reporting v2</t>
+        </is>
+      </c>
+      <c r="D11" s="75" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 15–16</t>
+        </is>
+      </c>
+      <c r="G11" s="76" t="inlineStr">
+        <is>
+          <t>📋 Planned</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Reporting v2 with charts, mobile-responsive, third-party integrations</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" s="69" t="inlineStr">
+        <is>
+          <t>v2.0.0</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>OneWork Enterprise</t>
+        </is>
+      </c>
+      <c r="D12" s="75" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Sprint 21–23</t>
+        </is>
+      </c>
+      <c r="G12" s="76" t="inlineStr">
+        <is>
+          <t>📋 Planned</t>
+        </is>
+      </c>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>AI-powered insights, advanced automation, enterprise scale</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr"/>
+      <c r="B14" s="13" t="n"/>
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
+      <c r="H14" s="14" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr"/>
+      <c r="B15" s="9" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="9" t="n"/>
+      <c r="F15" s="9" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="10" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr"/>
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="14" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr"/>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="F17" s="9" t="n"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="10" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr"/>
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="13" t="n"/>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="14" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A8:H8"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="008B5CF6"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Learn — Release History &amp; Roadmap 2026</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>All releases for Learn  •  Lead: Ricky  •  Team: Ricky, Loc, Than</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="30" t="inlineStr">
+        <is>
+          <t>Released: 1  •  Hotfixes: 0  •  Planned: 3  •  Latest: v1.0.0  •  Next: v1.1.0 (Jun 2026)</t>
+        </is>
+      </c>
+      <c r="B3" s="77" t="n"/>
+      <c r="C3" s="77" t="n"/>
+      <c r="D3" s="77" t="n"/>
+      <c r="E3" s="77" t="n"/>
+      <c r="F3" s="77" t="n"/>
+      <c r="G3" s="77" t="n"/>
+      <c r="H3" s="77" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="67" t="inlineStr">
+        <is>
+          <t>✅  RELEASED</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="31" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>Release Name</t>
+        </is>
+      </c>
+      <c r="D5" s="31" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E5" s="31" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F5" s="31" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="G5" s="31" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H5" s="31" t="inlineStr">
+        <is>
+          <t>Highlights / What's Included</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="69" t="inlineStr">
+        <is>
+          <t>v1.0.0</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Learn MVP</t>
+        </is>
+      </c>
+      <c r="D6" s="70" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>29 Mar 2026</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
+      </c>
+      <c r="G6" s="70" t="inlineStr">
+        <is>
+          <t>✅ Released</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>Courses, learning paths, assessments, certifications, progress tracking</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="73" t="inlineStr">
+        <is>
+          <t>📋  UPCOMING / PLANNED</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="n"/>
+      <c r="C8" s="60" t="n"/>
+      <c r="D8" s="60" t="n"/>
+      <c r="E8" s="60" t="n"/>
+      <c r="F8" s="60" t="n"/>
+      <c r="G8" s="60" t="n"/>
+      <c r="H8" s="60" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="74" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B9" s="74" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C9" s="74" t="inlineStr">
+        <is>
+          <t>Release Name</t>
+        </is>
+      </c>
+      <c r="D9" s="74" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E9" s="74" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F9" s="74" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="G9" s="74" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H9" s="74" t="inlineStr">
+        <is>
+          <t>Highlights / What's Included</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="69" t="inlineStr">
+        <is>
+          <t>v1.1.0</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>Learn Analytics</t>
+        </is>
+      </c>
+      <c r="D10" s="75" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Sprint 11–12</t>
+        </is>
+      </c>
+      <c r="G10" s="76" t="inlineStr">
+        <is>
+          <t>📋 Planned</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>Advanced analytics dashboard, learner recommendations, completion reports</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="71" t="inlineStr">
+        <is>
+          <t>v1.2.0</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Learn Marketplace</t>
+        </is>
+      </c>
+      <c r="D11" s="75" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 15–16</t>
+        </is>
+      </c>
+      <c r="G11" s="76" t="inlineStr">
+        <is>
+          <t>📋 Planned</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Content marketplace, SCORM support, mobile-responsive learning</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" s="69" t="inlineStr">
+        <is>
+          <t>v2.0.0</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>Learn Enterprise</t>
+        </is>
+      </c>
+      <c r="D12" s="75" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Sprint 21–23</t>
+        </is>
+      </c>
+      <c r="G12" s="76" t="inlineStr">
+        <is>
+          <t>📋 Planned</t>
+        </is>
+      </c>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>AI recommendations, adaptive learning, full mobile app</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr"/>
+      <c r="B14" s="13" t="n"/>
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
+      <c r="H14" s="14" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr"/>
+      <c r="B15" s="9" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="9" t="n"/>
+      <c r="F15" s="9" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="10" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr"/>
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="14" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr"/>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="F17" s="9" t="n"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="10" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr"/>
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="13" t="n"/>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="14" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A8:H8"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0010B981"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Safe — Release History &amp; Roadmap 2026</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>All releases for Safe  •  Lead: Faisal  •  Team: Faisal, Surya, Kiritini</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="23" t="inlineStr">
+        <is>
+          <t>Released: 1  •  Hotfixes: 0  •  Planned: 3  •  Latest: v1.0.0  •  Next: v1.1.0 (Jun 2026)</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n"/>
+      <c r="C3" s="7" t="n"/>
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="7" t="n"/>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="7" t="n"/>
+      <c r="H3" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="67" t="inlineStr">
+        <is>
+          <t>✅  RELEASED</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="40" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="40" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C5" s="40" t="inlineStr">
+        <is>
+          <t>Release Name</t>
+        </is>
+      </c>
+      <c r="D5" s="40" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E5" s="40" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F5" s="40" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="G5" s="40" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H5" s="40" t="inlineStr">
+        <is>
+          <t>Highlights / What's Included</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="69" t="inlineStr">
+        <is>
+          <t>v1.0.0</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Safe MVP</t>
+        </is>
+      </c>
+      <c r="D6" s="70" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>29 Mar 2026</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
+      </c>
+      <c r="G6" s="70" t="inlineStr">
+        <is>
+          <t>✅ Released</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>Policies, compliance tracking, audit workflows, risk matrix, dashboards</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="73" t="inlineStr">
+        <is>
+          <t>📋  UPCOMING / PLANNED</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="n"/>
+      <c r="C8" s="60" t="n"/>
+      <c r="D8" s="60" t="n"/>
+      <c r="E8" s="60" t="n"/>
+      <c r="F8" s="60" t="n"/>
+      <c r="G8" s="60" t="n"/>
+      <c r="H8" s="60" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="74" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B9" s="74" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C9" s="74" t="inlineStr">
+        <is>
+          <t>Release Name</t>
+        </is>
+      </c>
+      <c r="D9" s="74" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E9" s="74" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F9" s="74" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="G9" s="74" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H9" s="74" t="inlineStr">
+        <is>
+          <t>Highlights / What's Included</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="69" t="inlineStr">
+        <is>
+          <t>v1.1.0</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>Safe Regulatory Auto</t>
+        </is>
+      </c>
+      <c r="D10" s="75" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Sprint 11–12</t>
+        </is>
+      </c>
+      <c r="G10" s="76" t="inlineStr">
+        <is>
+          <t>📋 Planned</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>Regulatory update automation, scheduled compliance checks, advanced reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="71" t="inlineStr">
+        <is>
+          <t>v1.2.0</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Safe Integrations</t>
+        </is>
+      </c>
+      <c r="D11" s="75" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 17–18</t>
+        </is>
+      </c>
+      <c r="G11" s="76" t="inlineStr">
+        <is>
+          <t>📋 Planned</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Third-party GRC integrations, automated alerts, evidence collection</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" s="69" t="inlineStr">
+        <is>
+          <t>v2.0.0</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>Safe Enterprise</t>
+        </is>
+      </c>
+      <c r="D12" s="75" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Sprint 24–26</t>
+        </is>
+      </c>
+      <c r="G12" s="76" t="inlineStr">
+        <is>
+          <t>📋 Planned</t>
+        </is>
+      </c>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>Enterprise compliance suite with AI-driven risk predictions</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr"/>
+      <c r="B14" s="13" t="n"/>
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
+      <c r="H14" s="14" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr"/>
+      <c r="B15" s="9" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="9" t="n"/>
+      <c r="F15" s="9" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="10" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr"/>
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="14" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr"/>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="F17" s="9" t="n"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="10" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr"/>
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="13" t="n"/>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="14" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A8:H8"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00F59E0B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>OneHire — Release History &amp; Roadmap 2026</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>All releases for OneHire  •  Lead: Logesh  •  Team: Logesh, Hanis, Fatin, Sharuti</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="25" t="inlineStr">
+        <is>
+          <t>Released: 0  •  Hotfixes: 0  •  Planned: 3  •  Latest: —  •  Next: v0.1.0 (May 2026)</t>
+        </is>
+      </c>
+      <c r="B3" s="78" t="n"/>
+      <c r="C3" s="78" t="n"/>
+      <c r="D3" s="78" t="n"/>
+      <c r="E3" s="78" t="n"/>
+      <c r="F3" s="78" t="n"/>
+      <c r="G3" s="78" t="n"/>
+      <c r="H3" s="78" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="67" t="inlineStr">
+        <is>
+          <t>✅  RELEASED</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="45" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="45" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C5" s="45" t="inlineStr">
+        <is>
+          <t>Release Name</t>
+        </is>
+      </c>
+      <c r="D5" s="45" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E5" s="45" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F5" s="45" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="G5" s="45" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H5" s="45" t="inlineStr">
+        <is>
+          <t>Highlights / What's Included</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="79" t="inlineStr">
+        <is>
+          <t>No releases yet</t>
+        </is>
+      </c>
+      <c r="B6" s="80" t="n"/>
+      <c r="C6" s="80" t="n"/>
+      <c r="D6" s="80" t="n"/>
+      <c r="E6" s="80" t="n"/>
+      <c r="F6" s="80" t="n"/>
+      <c r="G6" s="80" t="n"/>
+      <c r="H6" s="80" t="n"/>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="73" t="inlineStr">
+        <is>
+          <t>📋  UPCOMING / PLANNED</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="n"/>
+      <c r="C8" s="60" t="n"/>
+      <c r="D8" s="60" t="n"/>
+      <c r="E8" s="60" t="n"/>
+      <c r="F8" s="60" t="n"/>
+      <c r="G8" s="60" t="n"/>
+      <c r="H8" s="60" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="74" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B9" s="74" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C9" s="74" t="inlineStr">
+        <is>
+          <t>Release Name</t>
+        </is>
+      </c>
+      <c r="D9" s="74" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E9" s="74" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F9" s="74" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="G9" s="74" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H9" s="74" t="inlineStr">
+        <is>
+          <t>Highlights / What's Included</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="69" t="inlineStr">
+        <is>
+          <t>v0.1.0</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>OneHire Alpha</t>
+        </is>
+      </c>
+      <c r="D10" s="81" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Sprint 9–10</t>
+        </is>
+      </c>
+      <c r="G10" s="76" t="inlineStr">
+        <is>
+          <t>📋 Planned</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>Core job posting and applicant tracking features</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="71" t="inlineStr">
+        <is>
+          <t>v0.5.0</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>OneHire Beta</t>
+        </is>
+      </c>
+      <c r="D11" s="81" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 11–12</t>
+        </is>
+      </c>
+      <c r="G11" s="76" t="inlineStr">
+        <is>
+          <t>📋 Planned</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Interview scheduling, candidate pipeline, basic reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" s="69" t="inlineStr">
+        <is>
+          <t>v1.0.0</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>OneHire MVP</t>
+        </is>
+      </c>
+      <c r="D12" s="70" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Sprint 13–14</t>
+        </is>
+      </c>
+      <c r="G12" s="76" t="inlineStr">
+        <is>
+          <t>📋 Planned</t>
+        </is>
+      </c>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>Full recruitment portal with applicant tracking and analytics</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr"/>
+      <c r="B14" s="13" t="n"/>
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
+      <c r="H14" s="14" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr"/>
+      <c r="B15" s="9" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="9" t="n"/>
+      <c r="F15" s="9" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="10" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr"/>
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="14" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr"/>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="F17" s="9" t="n"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="10" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr"/>
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="13" t="n"/>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="14" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A6:H6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00EF4444"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Spot — Release History &amp; Roadmap 2026</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>All releases for Spot  •  Lead: Ricky  •  Team: Ricky, Loc, Than, Majed, Hema</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>Released: 0  •  Hotfixes: 0  •  Planned: 2  •  Latest: —  •  Next: v0.1.0 (May 2026)</t>
+        </is>
+      </c>
+      <c r="B3" s="82" t="n"/>
+      <c r="C3" s="82" t="n"/>
+      <c r="D3" s="82" t="n"/>
+      <c r="E3" s="82" t="n"/>
+      <c r="F3" s="82" t="n"/>
+      <c r="G3" s="82" t="n"/>
+      <c r="H3" s="82" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="67" t="inlineStr">
+        <is>
+          <t>✅  RELEASED</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="48" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="48" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C5" s="48" t="inlineStr">
+        <is>
+          <t>Release Name</t>
+        </is>
+      </c>
+      <c r="D5" s="48" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E5" s="48" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F5" s="48" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="G5" s="48" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H5" s="48" t="inlineStr">
+        <is>
+          <t>Highlights / What's Included</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="79" t="inlineStr">
+        <is>
+          <t>No releases yet</t>
+        </is>
+      </c>
+      <c r="B6" s="80" t="n"/>
+      <c r="C6" s="80" t="n"/>
+      <c r="D6" s="80" t="n"/>
+      <c r="E6" s="80" t="n"/>
+      <c r="F6" s="80" t="n"/>
+      <c r="G6" s="80" t="n"/>
+      <c r="H6" s="80" t="n"/>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="73" t="inlineStr">
+        <is>
+          <t>📋  UPCOMING / PLANNED</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="n"/>
+      <c r="C8" s="60" t="n"/>
+      <c r="D8" s="60" t="n"/>
+      <c r="E8" s="60" t="n"/>
+      <c r="F8" s="60" t="n"/>
+      <c r="G8" s="60" t="n"/>
+      <c r="H8" s="60" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="74" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B9" s="74" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C9" s="74" t="inlineStr">
+        <is>
+          <t>Release Name</t>
+        </is>
+      </c>
+      <c r="D9" s="74" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E9" s="74" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F9" s="74" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="G9" s="74" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H9" s="74" t="inlineStr">
+        <is>
+          <t>Highlights / What's Included</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="69" t="inlineStr">
+        <is>
+          <t>v0.1.0</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>Spot Alpha</t>
+        </is>
+      </c>
+      <c r="D10" s="81" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Sprint 9–10</t>
+        </is>
+      </c>
+      <c r="G10" s="76" t="inlineStr">
+        <is>
+          <t>📋 Planned</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>Core city module, location management</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="71" t="inlineStr">
+        <is>
+          <t>v1.0.0</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Spot MVP</t>
+        </is>
+      </c>
+      <c r="D11" s="70" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 17–18</t>
+        </is>
+      </c>
+      <c r="G11" s="76" t="inlineStr">
+        <is>
+          <t>📋 Planned</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>City management, geolocation features, admin dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr"/>
+      <c r="B13" s="9" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="9" t="n"/>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="10" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr"/>
+      <c r="B14" s="13" t="n"/>
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
+      <c r="H14" s="14" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr"/>
+      <c r="B15" s="9" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="9" t="n"/>
+      <c r="F15" s="9" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="10" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr"/>
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="14" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr"/>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="F17" s="9" t="n"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="10" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A6:H6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00EC4899"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Pulse — Release History &amp; Roadmap 2026</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>All releases for Pulse  •  Lead: Hanis  •  Team: Hanis, Fatin, Majed, Hema, Rahmya, Umeshawar</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="26" t="inlineStr">
+        <is>
+          <t>Released: 0  •  Hotfixes: 0  •  Planned: 2  •  Latest: —  •  Next: v0.1.0 (May 2026)</t>
+        </is>
+      </c>
+      <c r="B3" s="83" t="n"/>
+      <c r="C3" s="83" t="n"/>
+      <c r="D3" s="83" t="n"/>
+      <c r="E3" s="83" t="n"/>
+      <c r="F3" s="83" t="n"/>
+      <c r="G3" s="83" t="n"/>
+      <c r="H3" s="83" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="67" t="inlineStr">
+        <is>
+          <t>✅  RELEASED</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="84" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="84" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C5" s="84" t="inlineStr">
+        <is>
+          <t>Release Name</t>
+        </is>
+      </c>
+      <c r="D5" s="84" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E5" s="84" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F5" s="84" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="G5" s="84" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H5" s="84" t="inlineStr">
+        <is>
+          <t>Highlights / What's Included</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="79" t="inlineStr">
+        <is>
+          <t>No releases yet</t>
+        </is>
+      </c>
+      <c r="B6" s="80" t="n"/>
+      <c r="C6" s="80" t="n"/>
+      <c r="D6" s="80" t="n"/>
+      <c r="E6" s="80" t="n"/>
+      <c r="F6" s="80" t="n"/>
+      <c r="G6" s="80" t="n"/>
+      <c r="H6" s="80" t="n"/>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="73" t="inlineStr">
+        <is>
+          <t>📋  UPCOMING / PLANNED</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="n"/>
+      <c r="C8" s="60" t="n"/>
+      <c r="D8" s="60" t="n"/>
+      <c r="E8" s="60" t="n"/>
+      <c r="F8" s="60" t="n"/>
+      <c r="G8" s="60" t="n"/>
+      <c r="H8" s="60" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="74" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B9" s="74" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C9" s="74" t="inlineStr">
+        <is>
+          <t>Release Name</t>
+        </is>
+      </c>
+      <c r="D9" s="74" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E9" s="74" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F9" s="74" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="G9" s="74" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H9" s="74" t="inlineStr">
+        <is>
+          <t>Highlights / What's Included</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="69" t="inlineStr">
+        <is>
+          <t>v0.1.0</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>Pulse Alpha</t>
+        </is>
+      </c>
+      <c r="D10" s="81" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Sprint 9–10</t>
+        </is>
+      </c>
+      <c r="G10" s="76" t="inlineStr">
+        <is>
+          <t>📋 Planned</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>Survey builder, basic distribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="71" t="inlineStr">
+        <is>
+          <t>v1.0.0</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Pulse MVP</t>
+        </is>
+      </c>
+      <c r="D11" s="70" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 17–18</t>
+        </is>
+      </c>
+      <c r="G11" s="76" t="inlineStr">
+        <is>
+          <t>📋 Planned</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Survey analytics, employee engagement dashboards, benchmarking</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr"/>
+      <c r="B13" s="9" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="9" t="n"/>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="10" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr"/>
+      <c r="B14" s="13" t="n"/>
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
+      <c r="H14" s="14" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr"/>
+      <c r="B15" s="9" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="9" t="n"/>
+      <c r="F15" s="9" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="10" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr"/>
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="14" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr"/>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="F17" s="9" t="n"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="10" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A6:H6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="000369A1"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -1385,14 +3669,14 @@
       <c r="D2" s="4" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="71" t="inlineStr">
+      <c r="A3" s="68" t="inlineStr">
         <is>
           <t>Versioning Format</t>
         </is>
       </c>
-      <c r="B3" s="72" t="n"/>
-      <c r="C3" s="72" t="n"/>
-      <c r="D3" s="73" t="n"/>
+      <c r="B3" s="85" t="n"/>
+      <c r="C3" s="85" t="n"/>
+      <c r="D3" s="86" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="49" t="inlineStr">
@@ -1400,13 +3684,13 @@
           <t>Format</t>
         </is>
       </c>
-      <c r="B4" s="74" t="inlineStr">
+      <c r="B4" s="87" t="inlineStr">
         <is>
           <t>vMAJOR.MINOR.PATCH</t>
         </is>
       </c>
-      <c r="C4" s="75" t="n"/>
-      <c r="D4" s="76" t="inlineStr">
+      <c r="C4" s="88" t="n"/>
+      <c r="D4" s="89" t="inlineStr">
         <is>
           <t>Example: v1.2.3</t>
         </is>
@@ -1418,13 +3702,13 @@
           <t>MAJOR</t>
         </is>
       </c>
-      <c r="B5" s="74" t="inlineStr">
+      <c r="B5" s="87" t="inlineStr">
         <is>
           <t>Breaking changes or major new feature sets</t>
         </is>
       </c>
-      <c r="C5" s="75" t="n"/>
-      <c r="D5" s="76" t="inlineStr">
+      <c r="C5" s="88" t="n"/>
+      <c r="D5" s="89" t="inlineStr">
         <is>
           <t>v1.0.0 → v2.0.0</t>
         </is>
@@ -1436,13 +3720,13 @@
           <t>MINOR</t>
         </is>
       </c>
-      <c r="B6" s="74" t="inlineStr">
+      <c r="B6" s="87" t="inlineStr">
         <is>
           <t>New features, enhancements (backward compatible)</t>
         </is>
       </c>
-      <c r="C6" s="75" t="n"/>
-      <c r="D6" s="76" t="inlineStr">
+      <c r="C6" s="88" t="n"/>
+      <c r="D6" s="89" t="inlineStr">
         <is>
           <t>v1.0.0 → v1.1.0</t>
         </is>
@@ -1454,13 +3738,13 @@
           <t>PATCH</t>
         </is>
       </c>
-      <c r="B7" s="74" t="inlineStr">
+      <c r="B7" s="87" t="inlineStr">
         <is>
           <t>Bug fixes, hotfixes, minor corrections</t>
         </is>
       </c>
-      <c r="C7" s="75" t="n"/>
-      <c r="D7" s="76" t="inlineStr">
+      <c r="C7" s="88" t="n"/>
+      <c r="D7" s="89" t="inlineStr">
         <is>
           <t>v1.0.0 → v1.0.1</t>
         </is>
@@ -1490,7 +3774,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="77" t="inlineStr">
+      <c r="A10" s="90" t="inlineStr">
         <is>
           <t>MVP</t>
         </is>
@@ -1512,7 +3796,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="78" t="inlineStr">
+      <c r="A11" s="91" t="inlineStr">
         <is>
           <t>Major</t>
         </is>
@@ -1534,7 +3818,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="79" t="inlineStr">
+      <c r="A12" s="92" t="inlineStr">
         <is>
           <t>Minor</t>
         </is>
@@ -1556,7 +3840,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="80" t="inlineStr">
+      <c r="A13" s="93" t="inlineStr">
         <is>
           <t>Hotfix</t>
         </is>
@@ -1578,7 +3862,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="81" t="inlineStr">
+      <c r="A14" s="94" t="inlineStr">
         <is>
           <t>Patch</t>
         </is>
@@ -1600,7 +3884,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="82" t="inlineStr">
+      <c r="A15" s="95" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
@@ -1623,122 +3907,122 @@
     </row>
     <row r="16"/>
     <row r="17">
-      <c r="A17" s="71" t="inlineStr">
+      <c r="A17" s="68" t="inlineStr">
         <is>
           <t>Release Naming Convention</t>
         </is>
       </c>
-      <c r="B17" s="72" t="n"/>
-      <c r="C17" s="72" t="n"/>
-      <c r="D17" s="73" t="n"/>
+      <c r="B17" s="85" t="n"/>
+      <c r="C17" s="85" t="n"/>
+      <c r="D17" s="86" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="83" t="inlineStr">
+      <c r="A18" s="96" t="inlineStr">
         <is>
           <t>Pattern</t>
         </is>
       </c>
-      <c r="B18" s="84" t="inlineStr">
+      <c r="B18" s="97" t="inlineStr">
         <is>
           <t>[Product] [Type] — [Short Description]</t>
         </is>
       </c>
-      <c r="C18" s="85" t="inlineStr">
+      <c r="C18" s="98" t="inlineStr">
         <is>
           <t>Used in Release Name column</t>
         </is>
       </c>
-      <c r="D18" s="86" t="n"/>
+      <c r="D18" s="99" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="83" t="inlineStr">
+      <c r="A19" s="96" t="inlineStr">
         <is>
           <t>MVP</t>
         </is>
       </c>
-      <c r="B19" s="84" t="inlineStr">
+      <c r="B19" s="97" t="inlineStr">
         <is>
           <t>AG ONE MVP</t>
         </is>
       </c>
-      <c r="C19" s="85" t="inlineStr">
+      <c r="C19" s="98" t="inlineStr">
         <is>
           <t>First production release</t>
         </is>
       </c>
-      <c r="D19" s="86" t="n"/>
+      <c r="D19" s="99" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="83" t="inlineStr">
+      <c r="A20" s="96" t="inlineStr">
         <is>
           <t>Minor</t>
         </is>
       </c>
-      <c r="B20" s="84" t="inlineStr">
+      <c r="B20" s="97" t="inlineStr">
         <is>
           <t>AG ONE Q2 Enhancement</t>
         </is>
       </c>
-      <c r="C20" s="85" t="inlineStr">
+      <c r="C20" s="98" t="inlineStr">
         <is>
           <t>Quarterly feature release</t>
         </is>
       </c>
-      <c r="D20" s="86" t="n"/>
+      <c r="D20" s="99" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="83" t="inlineStr">
+      <c r="A21" s="96" t="inlineStr">
         <is>
           <t>Hotfix</t>
         </is>
       </c>
-      <c r="B21" s="84" t="inlineStr">
+      <c r="B21" s="97" t="inlineStr">
         <is>
           <t>AG ONE Hotfix 1</t>
         </is>
       </c>
-      <c r="C21" s="85" t="inlineStr">
+      <c r="C21" s="98" t="inlineStr">
         <is>
           <t>Numbered sequentially</t>
         </is>
       </c>
-      <c r="D21" s="86" t="n"/>
+      <c r="D21" s="99" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="83" t="inlineStr">
+      <c r="A22" s="96" t="inlineStr">
         <is>
           <t>Major</t>
         </is>
       </c>
-      <c r="B22" s="84" t="inlineStr">
+      <c r="B22" s="97" t="inlineStr">
         <is>
           <t>AG ONE Enterprise</t>
         </is>
       </c>
-      <c r="C22" s="85" t="inlineStr">
+      <c r="C22" s="98" t="inlineStr">
         <is>
           <t>Named for the theme</t>
         </is>
       </c>
-      <c r="D22" s="86" t="n"/>
+      <c r="D22" s="99" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="83" t="inlineStr">
+      <c r="A23" s="96" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="B23" s="84" t="inlineStr">
+      <c r="B23" s="97" t="inlineStr">
         <is>
           <t>OneHire Alpha / OneHire Beta</t>
         </is>
       </c>
-      <c r="C23" s="85" t="inlineStr">
+      <c r="C23" s="98" t="inlineStr">
         <is>
           <t>Pre-MVP iterations</t>
         </is>
       </c>
-      <c r="D23" s="86" t="n"/>
+      <c r="D23" s="99" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -1762,7 +4046,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="006B7280"/>
@@ -1799,22 +4083,22 @@
       <c r="D2" s="4" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="71" t="inlineStr">
+      <c r="A3" s="68" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="B3" s="71" t="inlineStr">
+      <c r="B3" s="68" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="C3" s="71" t="inlineStr">
+      <c r="C3" s="68" t="inlineStr">
         <is>
           <t>Update Frequency</t>
         </is>
       </c>
-      <c r="D3" s="71" t="inlineStr">
+      <c r="D3" s="68" t="inlineStr">
         <is>
           <t>Who Updates</t>
         </is>
@@ -1999,12 +4283,12 @@
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>Release History</t>
+          <t>Rel-[Product]</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>Full log of every release: MVP, minor, major, hotfix, patch, sprint</t>
+          <t>Per-product release tab — released + upcoming with highlights (7 tabs)</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
@@ -2042,51 +4326,51 @@
     </row>
     <row r="14"/>
     <row r="15">
-      <c r="A15" s="87" t="inlineStr">
+      <c r="A15" s="100" t="inlineStr">
         <is>
           <t>STATUS LEGEND</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="88" t="inlineStr">
+      <c r="A16" s="101" t="inlineStr">
         <is>
           <t xml:space="preserve">  ●  ✅ Completed</t>
         </is>
       </c>
-      <c r="B16" s="73" t="n"/>
+      <c r="B16" s="86" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="89" t="inlineStr">
+      <c r="A17" s="102" t="inlineStr">
         <is>
           <t xml:space="preserve">  ●  ▶ In Progress / On Track</t>
         </is>
       </c>
-      <c r="B17" s="73" t="n"/>
+      <c r="B17" s="86" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="90" t="inlineStr">
+      <c r="A18" s="103" t="inlineStr">
         <is>
           <t xml:space="preserve">  ●  At Risk</t>
         </is>
       </c>
-      <c r="B18" s="73" t="n"/>
+      <c r="B18" s="86" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="91" t="inlineStr">
+      <c r="A19" s="104" t="inlineStr">
         <is>
           <t xml:space="preserve">  ●  Blocked</t>
         </is>
       </c>
-      <c r="B19" s="73" t="n"/>
+      <c r="B19" s="86" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="92" t="inlineStr">
+      <c r="A20" s="105" t="inlineStr">
         <is>
           <t xml:space="preserve">  ●  Not Started</t>
         </is>
       </c>
-      <c r="B20" s="73" t="n"/>
+      <c r="B20" s="86" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -10555,28 +12839,27 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="000284C7"/>
+    <tabColor rgb="001E3A5F"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="55" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Release History — Full Log 2026</t>
+          <t>AG ONE — Release History &amp; Roadmap 2026</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -10586,12 +12869,11 @@
       <c r="F1" s="2" t="n"/>
       <c r="G1" s="2" t="n"/>
       <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Every release across all products: MVP, minor, major, hotfix, patch, sprint releases</t>
+          <t>All releases for AG ONE  •  Lead: Geena  •  Team: Geena, Nastaran</t>
         </is>
       </c>
       <c r="B2" s="4" t="n"/>
@@ -10601,1314 +12883,432 @@
       <c r="F2" s="4" t="n"/>
       <c r="G2" s="4" t="n"/>
       <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="66" t="inlineStr">
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>Released: 3  •  Hotfixes: 2  •  Planned: 3  •  Latest: v1.0.2  •  Next: v1.1.0 (May 2026)</t>
+        </is>
+      </c>
+      <c r="B3" s="66" t="n"/>
+      <c r="C3" s="66" t="n"/>
+      <c r="D3" s="66" t="n"/>
+      <c r="E3" s="66" t="n"/>
+      <c r="F3" s="66" t="n"/>
+      <c r="G3" s="66" t="n"/>
+      <c r="H3" s="66" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="67" t="inlineStr">
+        <is>
+          <t>✅  RELEASED</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="68" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="66" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="C3" s="66" t="inlineStr">
+      <c r="B5" s="68" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="D3" s="66" t="inlineStr">
+      <c r="C5" s="68" t="inlineStr">
         <is>
           <t>Release Name</t>
         </is>
       </c>
-      <c r="E3" s="66" t="inlineStr">
+      <c r="D5" s="68" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="F3" s="66" t="inlineStr">
+      <c r="E5" s="68" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="G3" s="66" t="inlineStr">
+      <c r="F5" s="68" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="H3" s="66" t="inlineStr">
+      <c r="G5" s="68" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I3" s="66" t="inlineStr">
+      <c r="H5" s="68" t="inlineStr">
         <is>
           <t>Highlights / What's Included</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="13" t="n">
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="32" t="inlineStr">
-        <is>
-          <t>AG ONE</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="B6" s="69" t="inlineStr">
         <is>
           <t>v1.0.0</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>AG ONE MVP</t>
         </is>
       </c>
-      <c r="E4" s="67" t="inlineStr">
+      <c r="D6" s="70" t="inlineStr">
         <is>
           <t>MVP</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="E6" s="13" t="inlineStr">
         <is>
           <t>29 Mar 2026</t>
         </is>
       </c>
-      <c r="G4" s="13" t="inlineStr">
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="H4" s="11" t="inlineStr">
+      <c r="G6" s="70" t="inlineStr">
         <is>
           <t>✅ Released</t>
         </is>
       </c>
-      <c r="I4" s="14" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>Full IAM platform: Users, Roles, Tenants, SSO, Permissions, Audit, Assign Access</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="9" t="n">
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="32" t="inlineStr">
-        <is>
-          <t>AG ONE</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="B7" s="71" t="inlineStr">
         <is>
           <t>v1.0.1</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>AG ONE Hotfix 1</t>
         </is>
       </c>
-      <c r="E5" s="68" t="inlineStr">
+      <c r="D7" s="72" t="inlineStr">
         <is>
           <t>Hotfix</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>02 Apr 2026</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>Sprint 7</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr">
+      <c r="G7" s="70" t="inlineStr">
         <is>
           <t>✅ Released</t>
         </is>
       </c>
-      <c r="I5" s="10" t="inlineStr">
+      <c r="H7" s="10" t="inlineStr">
         <is>
           <t>SSO token refresh loop fix, role sync cache invalidation, tenant switching fix</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="13" t="n">
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="32" t="inlineStr">
-        <is>
-          <t>AG ONE</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="B8" s="69" t="inlineStr">
         <is>
           <t>v1.0.2</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>AG ONE Hotfix 2</t>
         </is>
       </c>
-      <c r="E6" s="68" t="inlineStr">
+      <c r="D8" s="72" t="inlineStr">
         <is>
           <t>Hotfix</t>
         </is>
       </c>
-      <c r="F6" s="13" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>08 Apr 2026</t>
         </is>
       </c>
-      <c r="G6" s="13" t="inlineStr">
+      <c r="F8" s="13" t="inlineStr">
         <is>
           <t>Sprint 7</t>
         </is>
       </c>
-      <c r="H6" s="11" t="inlineStr">
+      <c r="G8" s="70" t="inlineStr">
         <is>
           <t>✅ Released</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
+      <c r="H8" s="14" t="inlineStr">
         <is>
           <t>Audit log pagination, API key duplicate name validation, timezone fix</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="32" t="inlineStr">
-        <is>
-          <t>AG ONE</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="73" t="inlineStr">
+        <is>
+          <t>📋  UPCOMING / PLANNED</t>
+        </is>
+      </c>
+      <c r="B10" s="60" t="n"/>
+      <c r="C10" s="60" t="n"/>
+      <c r="D10" s="60" t="n"/>
+      <c r="E10" s="60" t="n"/>
+      <c r="F10" s="60" t="n"/>
+      <c r="G10" s="60" t="n"/>
+      <c r="H10" s="60" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="74" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B11" s="74" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C11" s="74" t="inlineStr">
+        <is>
+          <t>Release Name</t>
+        </is>
+      </c>
+      <c r="D11" s="74" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E11" s="74" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F11" s="74" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="G11" s="74" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H11" s="74" t="inlineStr">
+        <is>
+          <t>Highlights / What's Included</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="69" t="inlineStr">
         <is>
           <t>v1.1.0</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>AG ONE Q2 Enhancement</t>
         </is>
       </c>
-      <c r="E7" s="69" t="inlineStr">
+      <c r="D12" s="75" t="inlineStr">
         <is>
           <t>Minor</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="E12" s="13" t="inlineStr">
         <is>
           <t>May 2026</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>Sprint 9–10</t>
         </is>
       </c>
-      <c r="H7" s="18" t="inlineStr">
+      <c r="G12" s="76" t="inlineStr">
         <is>
           <t>📋 Planned</t>
         </is>
       </c>
-      <c r="I7" s="10" t="inlineStr">
+      <c r="H12" s="14" t="inlineStr">
         <is>
           <t>Advanced user analytics, bulk role operations, enhanced audit dashboard</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="32" t="inlineStr">
-        <is>
-          <t>AG ONE</t>
-        </is>
-      </c>
-      <c r="C8" s="13" t="inlineStr">
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="71" t="inlineStr">
         <is>
           <t>v1.2.0</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>AG ONE Multi-Product Admin</t>
         </is>
       </c>
-      <c r="E8" s="69" t="inlineStr">
+      <c r="D13" s="75" t="inlineStr">
         <is>
           <t>Minor</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>Jul 2026</t>
         </is>
       </c>
-      <c r="G8" s="13" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>Sprint 13–14</t>
         </is>
       </c>
-      <c r="H8" s="18" t="inlineStr">
+      <c r="G13" s="76" t="inlineStr">
         <is>
           <t>📋 Planned</t>
         </is>
       </c>
-      <c r="I8" s="14" t="inlineStr">
+      <c r="H13" s="10" t="inlineStr">
         <is>
           <t>Multi-product admin console, cross-product role mapping, API marketplace v1</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="32" t="inlineStr">
-        <is>
-          <t>AG ONE</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" s="69" t="inlineStr">
         <is>
           <t>v2.0.0</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>AG ONE Enterprise</t>
         </is>
       </c>
-      <c r="E9" s="69" t="inlineStr">
+      <c r="D14" s="75" t="inlineStr">
         <is>
           <t>Major</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="E14" s="13" t="inlineStr">
         <is>
           <t>Oct 2026</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="F14" s="13" t="inlineStr">
         <is>
           <t>Sprint 20–22</t>
         </is>
       </c>
-      <c r="H9" s="18" t="inlineStr">
+      <c r="G14" s="76" t="inlineStr">
         <is>
           <t>📋 Planned</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr">
+      <c r="H14" s="14" t="inlineStr">
         <is>
           <t>Enterprise SSO (SAML+OIDC), advanced RBAC, white-label branding, scale</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="34" t="inlineStr">
-        <is>
-          <t>OneWork</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>v1.0.0</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>OneWork MVP</t>
-        </is>
-      </c>
-      <c r="E10" s="67" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
-        <is>
-          <t>29 Mar 2026</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 6</t>
-        </is>
-      </c>
-      <c r="H10" s="11" t="inlineStr">
-        <is>
-          <t>✅ Released</t>
-        </is>
-      </c>
-      <c r="I10" s="14" t="inlineStr">
-        <is>
-          <t>Employee mgmt, workflows, task mgmt, dashboards, reporting</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="34" t="inlineStr">
-        <is>
-          <t>OneWork</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>v1.1.0</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>OneWork Q2 Enhancement</t>
-        </is>
-      </c>
-      <c r="E11" s="69" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>Jun 2026</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 11–12</t>
-        </is>
-      </c>
-      <c r="H11" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I11" s="10" t="inlineStr">
-        <is>
-          <t>Advanced workflow templates, email notifications, calendar integration</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="13" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="34" t="inlineStr">
-        <is>
-          <t>OneWork</t>
-        </is>
-      </c>
-      <c r="C12" s="13" t="inlineStr">
-        <is>
-          <t>v1.2.0</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>OneWork Reporting v2</t>
-        </is>
-      </c>
-      <c r="E12" s="69" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
-        <is>
-          <t>Aug 2026</t>
-        </is>
-      </c>
-      <c r="G12" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 15–16</t>
-        </is>
-      </c>
-      <c r="H12" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I12" s="14" t="inlineStr">
-        <is>
-          <t>Reporting v2 with charts, mobile-responsive, third-party integrations</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="B13" s="34" t="inlineStr">
-        <is>
-          <t>OneWork</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>v2.0.0</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>OneWork Enterprise</t>
-        </is>
-      </c>
-      <c r="E13" s="69" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>Nov 2026</t>
-        </is>
-      </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 21–23</t>
-        </is>
-      </c>
-      <c r="H13" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I13" s="10" t="inlineStr">
-        <is>
-          <t>AI-powered insights, advanced automation, enterprise scale</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="n">
-        <v>11</v>
-      </c>
-      <c r="B14" s="35" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="C14" s="13" t="inlineStr">
-        <is>
-          <t>v1.0.0</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>Learn MVP</t>
-        </is>
-      </c>
-      <c r="E14" s="67" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="F14" s="13" t="inlineStr">
-        <is>
-          <t>29 Mar 2026</t>
-        </is>
-      </c>
-      <c r="G14" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 6</t>
-        </is>
-      </c>
-      <c r="H14" s="11" t="inlineStr">
-        <is>
-          <t>✅ Released</t>
-        </is>
-      </c>
-      <c r="I14" s="14" t="inlineStr">
-        <is>
-          <t>Courses, learning paths, assessments, certifications, progress tracking</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="B15" s="35" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>v1.1.0</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>Learn Analytics</t>
-        </is>
-      </c>
-      <c r="E15" s="69" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>Jun 2026</t>
-        </is>
-      </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 11–12</t>
-        </is>
-      </c>
-      <c r="H15" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I15" s="10" t="inlineStr">
-        <is>
-          <t>Advanced analytics dashboard, learner recommendations, completion reports</t>
-        </is>
-      </c>
-    </row>
+    <row r="15"/>
     <row r="16">
-      <c r="A16" s="13" t="n">
-        <v>13</v>
-      </c>
-      <c r="B16" s="35" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="C16" s="13" t="inlineStr">
-        <is>
-          <t>v1.2.0</t>
-        </is>
-      </c>
-      <c r="D16" s="14" t="inlineStr">
-        <is>
-          <t>Learn Marketplace</t>
-        </is>
-      </c>
-      <c r="E16" s="69" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="F16" s="13" t="inlineStr">
-        <is>
-          <t>Aug 2026</t>
-        </is>
-      </c>
-      <c r="G16" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 15–16</t>
-        </is>
-      </c>
-      <c r="H16" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I16" s="14" t="inlineStr">
-        <is>
-          <t>Content marketplace, SCORM support, mobile-responsive learning</t>
-        </is>
-      </c>
+      <c r="A16" s="13" t="inlineStr"/>
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="14" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="n">
-        <v>14</v>
-      </c>
-      <c r="B17" s="35" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>v2.0.0</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>Learn Enterprise</t>
-        </is>
-      </c>
-      <c r="E17" s="69" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>Nov 2026</t>
-        </is>
-      </c>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 21–23</t>
-        </is>
-      </c>
-      <c r="H17" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I17" s="10" t="inlineStr">
-        <is>
-          <t>AI recommendations, adaptive learning, full mobile app</t>
-        </is>
-      </c>
+      <c r="A17" s="9" t="inlineStr"/>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="F17" s="9" t="n"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="10" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="n">
-        <v>15</v>
-      </c>
-      <c r="B18" s="36" t="inlineStr">
-        <is>
-          <t>Safe</t>
-        </is>
-      </c>
-      <c r="C18" s="13" t="inlineStr">
-        <is>
-          <t>v1.0.0</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>Safe MVP</t>
-        </is>
-      </c>
-      <c r="E18" s="67" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
-        <is>
-          <t>29 Mar 2026</t>
-        </is>
-      </c>
-      <c r="G18" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 6</t>
-        </is>
-      </c>
-      <c r="H18" s="11" t="inlineStr">
-        <is>
-          <t>✅ Released</t>
-        </is>
-      </c>
-      <c r="I18" s="14" t="inlineStr">
-        <is>
-          <t>Policies, compliance tracking, audit workflows, risk matrix, dashboards</t>
-        </is>
-      </c>
+      <c r="A18" s="13" t="inlineStr"/>
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="13" t="n"/>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="14" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="n">
-        <v>16</v>
-      </c>
-      <c r="B19" s="36" t="inlineStr">
-        <is>
-          <t>Safe</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>v1.1.0</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>Safe Regulatory Auto</t>
-        </is>
-      </c>
-      <c r="E19" s="69" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="F19" s="9" t="inlineStr">
-        <is>
-          <t>Jun 2026</t>
-        </is>
-      </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 11–12</t>
-        </is>
-      </c>
-      <c r="H19" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I19" s="10" t="inlineStr">
-        <is>
-          <t>Regulatory update automation, scheduled compliance checks, advanced reporting</t>
-        </is>
-      </c>
+      <c r="A19" s="9" t="inlineStr"/>
+      <c r="B19" s="9" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="9" t="n"/>
+      <c r="E19" s="9" t="n"/>
+      <c r="F19" s="9" t="n"/>
+      <c r="G19" s="9" t="n"/>
+      <c r="H19" s="10" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="n">
-        <v>17</v>
-      </c>
-      <c r="B20" s="36" t="inlineStr">
-        <is>
-          <t>Safe</t>
-        </is>
-      </c>
-      <c r="C20" s="13" t="inlineStr">
-        <is>
-          <t>v1.2.0</t>
-        </is>
-      </c>
-      <c r="D20" s="14" t="inlineStr">
-        <is>
-          <t>Safe Integrations</t>
-        </is>
-      </c>
-      <c r="E20" s="69" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-      <c r="G20" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 17–18</t>
-        </is>
-      </c>
-      <c r="H20" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I20" s="14" t="inlineStr">
-        <is>
-          <t>Third-party GRC integrations, automated alerts, evidence collection</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="n">
-        <v>18</v>
-      </c>
-      <c r="B21" s="36" t="inlineStr">
-        <is>
-          <t>Safe</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>v2.0.0</t>
-        </is>
-      </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>Safe Enterprise</t>
-        </is>
-      </c>
-      <c r="E21" s="69" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>Dec 2026</t>
-        </is>
-      </c>
-      <c r="G21" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 24–26</t>
-        </is>
-      </c>
-      <c r="H21" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I21" s="10" t="inlineStr">
-        <is>
-          <t>Enterprise compliance suite with AI-driven risk predictions</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="13" t="n">
-        <v>19</v>
-      </c>
-      <c r="B22" s="37" t="inlineStr">
-        <is>
-          <t>OneHire</t>
-        </is>
-      </c>
-      <c r="C22" s="13" t="inlineStr">
-        <is>
-          <t>v0.1.0</t>
-        </is>
-      </c>
-      <c r="D22" s="14" t="inlineStr">
-        <is>
-          <t>OneHire Alpha</t>
-        </is>
-      </c>
-      <c r="E22" s="70" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
-        <is>
-          <t>May 2026</t>
-        </is>
-      </c>
-      <c r="G22" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 9–10</t>
-        </is>
-      </c>
-      <c r="H22" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I22" s="14" t="inlineStr">
-        <is>
-          <t>Core job posting and applicant tracking features</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="B23" s="37" t="inlineStr">
-        <is>
-          <t>OneHire</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>v0.5.0</t>
-        </is>
-      </c>
-      <c r="D23" s="10" t="inlineStr">
-        <is>
-          <t>OneHire Beta</t>
-        </is>
-      </c>
-      <c r="E23" s="70" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>Jun 2026</t>
-        </is>
-      </c>
-      <c r="G23" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 11–12</t>
-        </is>
-      </c>
-      <c r="H23" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I23" s="10" t="inlineStr">
-        <is>
-          <t>Interview scheduling, candidate pipeline, basic reporting</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="13" t="n">
-        <v>21</v>
-      </c>
-      <c r="B24" s="37" t="inlineStr">
-        <is>
-          <t>OneHire</t>
-        </is>
-      </c>
-      <c r="C24" s="13" t="inlineStr">
-        <is>
-          <t>v1.0.0</t>
-        </is>
-      </c>
-      <c r="D24" s="14" t="inlineStr">
-        <is>
-          <t>OneHire MVP</t>
-        </is>
-      </c>
-      <c r="E24" s="67" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
-        <is>
-          <t>Jul 2026</t>
-        </is>
-      </c>
-      <c r="G24" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 13–14</t>
-        </is>
-      </c>
-      <c r="H24" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I24" s="14" t="inlineStr">
-        <is>
-          <t>Full recruitment portal with applicant tracking and analytics</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="B25" s="38" t="inlineStr">
-        <is>
-          <t>Spot</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>v0.1.0</t>
-        </is>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
-        <is>
-          <t>Spot Alpha</t>
-        </is>
-      </c>
-      <c r="E25" s="70" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="F25" s="9" t="inlineStr">
-        <is>
-          <t>May 2026</t>
-        </is>
-      </c>
-      <c r="G25" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 9–10</t>
-        </is>
-      </c>
-      <c r="H25" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I25" s="10" t="inlineStr">
-        <is>
-          <t>Core city module, location management</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="13" t="n">
-        <v>23</v>
-      </c>
-      <c r="B26" s="38" t="inlineStr">
-        <is>
-          <t>Spot</t>
-        </is>
-      </c>
-      <c r="C26" s="13" t="inlineStr">
-        <is>
-          <t>v1.0.0</t>
-        </is>
-      </c>
-      <c r="D26" s="14" t="inlineStr">
-        <is>
-          <t>Spot MVP</t>
-        </is>
-      </c>
-      <c r="E26" s="67" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="F26" s="13" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-      <c r="G26" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 17–18</t>
-        </is>
-      </c>
-      <c r="H26" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I26" s="14" t="inlineStr">
-        <is>
-          <t>City management, geolocation features, admin dashboard</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="n">
-        <v>24</v>
-      </c>
-      <c r="B27" s="39" t="inlineStr">
-        <is>
-          <t>Pulse</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>v0.1.0</t>
-        </is>
-      </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>Pulse Alpha</t>
-        </is>
-      </c>
-      <c r="E27" s="70" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="F27" s="9" t="inlineStr">
-        <is>
-          <t>May 2026</t>
-        </is>
-      </c>
-      <c r="G27" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 9–10</t>
-        </is>
-      </c>
-      <c r="H27" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I27" s="10" t="inlineStr">
-        <is>
-          <t>Survey builder, basic distribution</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="13" t="n">
-        <v>25</v>
-      </c>
-      <c r="B28" s="39" t="inlineStr">
-        <is>
-          <t>Pulse</t>
-        </is>
-      </c>
-      <c r="C28" s="13" t="inlineStr">
-        <is>
-          <t>v1.0.0</t>
-        </is>
-      </c>
-      <c r="D28" s="14" t="inlineStr">
-        <is>
-          <t>Pulse MVP</t>
-        </is>
-      </c>
-      <c r="E28" s="67" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-      <c r="G28" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 17–18</t>
-        </is>
-      </c>
-      <c r="H28" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I28" s="14" t="inlineStr">
-        <is>
-          <t>Survey analytics, employee engagement dashboards, benchmarking</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="B29" s="9" t="n"/>
-      <c r="C29" s="9" t="n"/>
-      <c r="D29" s="10" t="n"/>
-      <c r="E29" s="9" t="n"/>
-      <c r="F29" s="9" t="n"/>
-      <c r="G29" s="9" t="n"/>
-      <c r="H29" s="9" t="n"/>
-      <c r="I29" s="10" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="13" t="n">
-        <v>27</v>
-      </c>
-      <c r="B30" s="13" t="n"/>
-      <c r="C30" s="13" t="n"/>
-      <c r="D30" s="14" t="n"/>
-      <c r="E30" s="13" t="n"/>
-      <c r="F30" s="13" t="n"/>
-      <c r="G30" s="13" t="n"/>
-      <c r="H30" s="13" t="n"/>
-      <c r="I30" s="14" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="n">
-        <v>28</v>
-      </c>
-      <c r="B31" s="9" t="n"/>
-      <c r="C31" s="9" t="n"/>
-      <c r="D31" s="10" t="n"/>
-      <c r="E31" s="9" t="n"/>
-      <c r="F31" s="9" t="n"/>
-      <c r="G31" s="9" t="n"/>
-      <c r="H31" s="9" t="n"/>
-      <c r="I31" s="10" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="13" t="n">
-        <v>29</v>
-      </c>
-      <c r="B32" s="13" t="n"/>
-      <c r="C32" s="13" t="n"/>
-      <c r="D32" s="14" t="n"/>
-      <c r="E32" s="13" t="n"/>
-      <c r="F32" s="13" t="n"/>
-      <c r="G32" s="13" t="n"/>
-      <c r="H32" s="13" t="n"/>
-      <c r="I32" s="14" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="B33" s="9" t="n"/>
-      <c r="C33" s="9" t="n"/>
-      <c r="D33" s="10" t="n"/>
-      <c r="E33" s="9" t="n"/>
-      <c r="F33" s="9" t="n"/>
-      <c r="G33" s="9" t="n"/>
-      <c r="H33" s="9" t="n"/>
-      <c r="I33" s="10" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="13" t="n">
-        <v>31</v>
-      </c>
-      <c r="B34" s="13" t="n"/>
-      <c r="C34" s="13" t="n"/>
-      <c r="D34" s="14" t="n"/>
-      <c r="E34" s="13" t="n"/>
-      <c r="F34" s="13" t="n"/>
-      <c r="G34" s="13" t="n"/>
-      <c r="H34" s="13" t="n"/>
-      <c r="I34" s="14" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="9" t="n">
-        <v>32</v>
-      </c>
-      <c r="B35" s="9" t="n"/>
-      <c r="C35" s="9" t="n"/>
-      <c r="D35" s="10" t="n"/>
-      <c r="E35" s="9" t="n"/>
-      <c r="F35" s="9" t="n"/>
-      <c r="G35" s="9" t="n"/>
-      <c r="H35" s="9" t="n"/>
-      <c r="I35" s="10" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="13" t="n">
-        <v>33</v>
-      </c>
-      <c r="B36" s="13" t="n"/>
-      <c r="C36" s="13" t="n"/>
-      <c r="D36" s="14" t="n"/>
-      <c r="E36" s="13" t="n"/>
-      <c r="F36" s="13" t="n"/>
-      <c r="G36" s="13" t="n"/>
-      <c r="H36" s="13" t="n"/>
-      <c r="I36" s="14" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="9" t="n">
-        <v>34</v>
-      </c>
-      <c r="B37" s="9" t="n"/>
-      <c r="C37" s="9" t="n"/>
-      <c r="D37" s="10" t="n"/>
-      <c r="E37" s="9" t="n"/>
-      <c r="F37" s="9" t="n"/>
-      <c r="G37" s="9" t="n"/>
-      <c r="H37" s="9" t="n"/>
-      <c r="I37" s="10" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="13" t="n">
-        <v>35</v>
-      </c>
-      <c r="B38" s="13" t="n"/>
-      <c r="C38" s="13" t="n"/>
-      <c r="D38" s="14" t="n"/>
-      <c r="E38" s="13" t="n"/>
-      <c r="F38" s="13" t="n"/>
-      <c r="G38" s="13" t="n"/>
-      <c r="H38" s="13" t="n"/>
-      <c r="I38" s="14" t="n"/>
+      <c r="A20" s="13" t="inlineStr"/>
+      <c r="B20" s="13" t="n"/>
+      <c r="C20" s="14" t="n"/>
+      <c r="D20" s="13" t="n"/>
+      <c r="E20" s="13" t="n"/>
+      <c r="F20" s="13" t="n"/>
+      <c r="G20" s="13" t="n"/>
+      <c r="H20" s="14" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+  <mergeCells count="5">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>

</xml_diff>

<commit_message>
Separate release tracking into its own Excel file
New file: AG_ONE_Release_History.xlsx (9 sheets)
- Release Dashboard: all products summary
- Per-product tabs: AG ONE, OneWork, Learn, Safe, OneHire, Spot, Pulse
  Each has: stats banner, Released section, Upcoming section, blank rows
- Release Standard: versioning policy + naming convention

Team Tracker cleaned: AG_ONE_Team_Tracker_2026.xlsx (8 sheets)
- Removed release sheets — now purely team/resource/sprint focused
- Team Overview, Resource Allocation, Project Roadmap, Sprint Tracker,
  Member Performance, 2026 Targets, External Projects, How To Use

Generator: create_release_tracker.py (new, standalone)

Co-authored-by: zainabbastahirag <zainabbastahirag@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AG_ONE_Team_Tracker_2026.xlsx
+++ b/AG_ONE_Team_Tracker_2026.xlsx
@@ -14,10 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Member Performance" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Targets" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External Projects" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Dashboard" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release History" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Standard" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How To Use" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How To Use" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="29">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -138,50 +135,14 @@
     <font>
       <name val="Aptos"/>
       <b val="1"/>
-      <color rgb="000369A1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <b val="1"/>
-      <color rgb="00065F46"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <b val="1"/>
-      <color rgb="00991B1B"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <b val="1"/>
-      <color rgb="00991B1B"/>
+      <color rgb="001E3A5F"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <b val="1"/>
-      <color rgb="006B7280"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Aptos"/>
       <b val="1"/>
       <color rgb="001E3A5F"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <b val="1"/>
-      <color rgb="005B21B6"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <b val="1"/>
-      <color rgb="001E3A5F"/>
-      <sz val="12"/>
     </font>
     <font>
       <name val="Aptos"/>
@@ -202,7 +163,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -305,26 +266,8 @@
         <bgColor rgb="00EDE9FE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="000EA5E9"/>
-        <bgColor rgb="000EA5E9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E0F2FE"/>
-        <bgColor rgb="00E0F2FE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00475569"/>
-        <bgColor rgb="00475569"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="6">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -368,17 +311,6 @@
     </border>
     <border>
       <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00E2E8F0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00E2E8F0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color rgb="00E2E8F0"/>
       </right>
@@ -394,7 +326,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -547,124 +479,16 @@
     <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="16" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1379,761 +1203,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="000369A1"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Release Naming Standard &amp; Versioning Policy</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Share this with all teams so everyone follows the same release naming and numbering</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="86" t="inlineStr">
-        <is>
-          <t>Versioning Format</t>
-        </is>
-      </c>
-      <c r="B3" s="87" t="n"/>
-      <c r="C3" s="87" t="n"/>
-      <c r="D3" s="88" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="49" t="inlineStr">
-        <is>
-          <t>Format</t>
-        </is>
-      </c>
-      <c r="B4" s="89" t="inlineStr">
-        <is>
-          <t>vMAJOR.MINOR.PATCH</t>
-        </is>
-      </c>
-      <c r="C4" s="90" t="n"/>
-      <c r="D4" s="91" t="inlineStr">
-        <is>
-          <t>Example: v1.2.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="49" t="inlineStr">
-        <is>
-          <t>MAJOR</t>
-        </is>
-      </c>
-      <c r="B5" s="89" t="inlineStr">
-        <is>
-          <t>Breaking changes or major new feature sets</t>
-        </is>
-      </c>
-      <c r="C5" s="90" t="n"/>
-      <c r="D5" s="91" t="inlineStr">
-        <is>
-          <t>v1.0.0 → v2.0.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="49" t="inlineStr">
-        <is>
-          <t>MINOR</t>
-        </is>
-      </c>
-      <c r="B6" s="89" t="inlineStr">
-        <is>
-          <t>New features, enhancements (backward compatible)</t>
-        </is>
-      </c>
-      <c r="C6" s="90" t="n"/>
-      <c r="D6" s="91" t="inlineStr">
-        <is>
-          <t>v1.0.0 → v1.1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="49" t="inlineStr">
-        <is>
-          <t>PATCH</t>
-        </is>
-      </c>
-      <c r="B7" s="89" t="inlineStr">
-        <is>
-          <t>Bug fixes, hotfixes, minor corrections</t>
-        </is>
-      </c>
-      <c r="C7" s="90" t="n"/>
-      <c r="D7" s="91" t="inlineStr">
-        <is>
-          <t>v1.0.0 → v1.0.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" s="58" t="inlineStr">
-        <is>
-          <t>Release Type</t>
-        </is>
-      </c>
-      <c r="B9" s="58" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C9" s="58" t="inlineStr">
-        <is>
-          <t>Frequency</t>
-        </is>
-      </c>
-      <c r="D9" s="58" t="inlineStr">
-        <is>
-          <t>Approval</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="92" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="B10" s="50" t="inlineStr">
-        <is>
-          <t>First production release of a product</t>
-        </is>
-      </c>
-      <c r="C10" s="50" t="inlineStr">
-        <is>
-          <t>Once per product</t>
-        </is>
-      </c>
-      <c r="D10" s="50" t="inlineStr">
-        <is>
-          <t>Director + Tech Lead</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="93" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="B11" s="50" t="inlineStr">
-        <is>
-          <t>Significant new features or breaking changes</t>
-        </is>
-      </c>
-      <c r="C11" s="50" t="inlineStr">
-        <is>
-          <t>1–2 per year</t>
-        </is>
-      </c>
-      <c r="D11" s="50" t="inlineStr">
-        <is>
-          <t>Director + Tech Lead</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="94" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="B12" s="50" t="inlineStr">
-        <is>
-          <t>New features &amp; enhancements, backward compatible</t>
-        </is>
-      </c>
-      <c r="C12" s="50" t="inlineStr">
-        <is>
-          <t>Quarterly</t>
-        </is>
-      </c>
-      <c r="D12" s="50" t="inlineStr">
-        <is>
-          <t>Tech Lead</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="95" t="inlineStr">
-        <is>
-          <t>Hotfix</t>
-        </is>
-      </c>
-      <c r="B13" s="50" t="inlineStr">
-        <is>
-          <t>Critical production fix, expedited deployment</t>
-        </is>
-      </c>
-      <c r="C13" s="50" t="inlineStr">
-        <is>
-          <t>As needed (urgent)</t>
-        </is>
-      </c>
-      <c r="D13" s="50" t="inlineStr">
-        <is>
-          <t>Tech Lead + post-mortem</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="96" t="inlineStr">
-        <is>
-          <t>Patch</t>
-        </is>
-      </c>
-      <c r="B14" s="50" t="inlineStr">
-        <is>
-          <t>Non-critical bug fixes, scheduled deployment</t>
-        </is>
-      </c>
-      <c r="C14" s="50" t="inlineStr">
-        <is>
-          <t>As needed</t>
-        </is>
-      </c>
-      <c r="D14" s="50" t="inlineStr">
-        <is>
-          <t>Tech Lead</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="97" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="B15" s="50" t="inlineStr">
-        <is>
-          <t>Sprint-based release (pre-MVP iterations)</t>
-        </is>
-      </c>
-      <c r="C15" s="50" t="inlineStr">
-        <is>
-          <t>Every 2 weeks</t>
-        </is>
-      </c>
-      <c r="D15" s="50" t="inlineStr">
-        <is>
-          <t>Tech Lead</t>
-        </is>
-      </c>
-    </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="86" t="inlineStr">
-        <is>
-          <t>Release Naming Convention</t>
-        </is>
-      </c>
-      <c r="B17" s="87" t="n"/>
-      <c r="C17" s="87" t="n"/>
-      <c r="D17" s="88" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="98" t="inlineStr">
-        <is>
-          <t>Pattern</t>
-        </is>
-      </c>
-      <c r="B18" s="99" t="inlineStr">
-        <is>
-          <t>[Product] [Type] — [Short Description]</t>
-        </is>
-      </c>
-      <c r="C18" s="100" t="inlineStr">
-        <is>
-          <t>Used in Release Name column</t>
-        </is>
-      </c>
-      <c r="D18" s="101" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="98" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="B19" s="99" t="inlineStr">
-        <is>
-          <t>AG ONE MVP</t>
-        </is>
-      </c>
-      <c r="C19" s="100" t="inlineStr">
-        <is>
-          <t>First production release</t>
-        </is>
-      </c>
-      <c r="D19" s="101" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="98" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="B20" s="99" t="inlineStr">
-        <is>
-          <t>AG ONE Q2 Enhancement</t>
-        </is>
-      </c>
-      <c r="C20" s="100" t="inlineStr">
-        <is>
-          <t>Quarterly feature release</t>
-        </is>
-      </c>
-      <c r="D20" s="101" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="98" t="inlineStr">
-        <is>
-          <t>Hotfix</t>
-        </is>
-      </c>
-      <c r="B21" s="99" t="inlineStr">
-        <is>
-          <t>AG ONE Hotfix 1</t>
-        </is>
-      </c>
-      <c r="C21" s="100" t="inlineStr">
-        <is>
-          <t>Numbered sequentially</t>
-        </is>
-      </c>
-      <c r="D21" s="101" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="98" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="B22" s="99" t="inlineStr">
-        <is>
-          <t>AG ONE Enterprise</t>
-        </is>
-      </c>
-      <c r="C22" s="100" t="inlineStr">
-        <is>
-          <t>Named for the theme</t>
-        </is>
-      </c>
-      <c r="D22" s="101" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="98" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="B23" s="99" t="inlineStr">
-        <is>
-          <t>OneHire Alpha / OneHire Beta</t>
-        </is>
-      </c>
-      <c r="C23" s="100" t="inlineStr">
-        <is>
-          <t>Pre-MVP iterations</t>
-        </is>
-      </c>
-      <c r="D23" s="101" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="B4:C4"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="006B7280"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>How To Use This Tracker</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Quick guide for all stakeholders</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="86" t="inlineStr">
-        <is>
-          <t>Sheet</t>
-        </is>
-      </c>
-      <c r="B3" s="86" t="inlineStr">
-        <is>
-          <t>Purpose</t>
-        </is>
-      </c>
-      <c r="C3" s="86" t="inlineStr">
-        <is>
-          <t>Update Frequency</t>
-        </is>
-      </c>
-      <c r="D3" s="86" t="inlineStr">
-        <is>
-          <t>Who Updates</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="13" t="inlineStr">
-        <is>
-          <t>Team Overview</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>See all 7 internal teams, current sprint, status at a glance</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>Every sprint</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>Engineering Manager</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Resource Allocation</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>Internal + external assignments per member, shared &amp; outsource flags</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>When team changes</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>Engineering Manager</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>Project Roadmap</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>Track project start/end, achievements, next targets, alignment</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="inlineStr">
-        <is>
-          <t>Every sprint</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Tech Leads</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>Sprint Tracker</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>Detailed sprint goals, outcomes, tech lead feedback, blockers</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>Every sprint</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>Tech Leads</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>Member Performance</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>Individual progress, ratings, achievements</t>
-        </is>
-      </c>
-      <c r="C8" s="13" t="inlineStr">
-        <is>
-          <t>Every sprint</t>
-        </is>
-      </c>
-      <c r="D8" s="13" t="inlineStr">
-        <is>
-          <t>Tech Leads</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>2026 Targets</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>Quarterly milestones and year-end goals per team</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Quarterly</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>Engineering Manager</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="13" t="inlineStr">
-        <is>
-          <t>External Projects</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>Track resources on external / outsource / partner projects</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>When assignments change</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>Engineering Manager</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>Release Dashboard</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>At-a-glance: latest release, totals, and next planned per product</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>Every release</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Engineering Manager</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>Release History</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>All releases grouped by product — released + upcoming with highlights</t>
-        </is>
-      </c>
-      <c r="C12" s="13" t="inlineStr">
-        <is>
-          <t>Every release</t>
-        </is>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>Tech Leads</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>Release Standard</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Versioning policy, naming convention, release types — share with all teams</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>Reference only</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="14"/>
-    <row r="15">
-      <c r="A15" s="102" t="inlineStr">
-        <is>
-          <t>STATUS LEGEND</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ●  ✅ Completed</t>
-        </is>
-      </c>
-      <c r="B16" s="88" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="104" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ●  ▶ In Progress / On Track</t>
-        </is>
-      </c>
-      <c r="B17" s="88" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="105" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ●  At Risk</t>
-        </is>
-      </c>
-      <c r="B18" s="88" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="106" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ●  Blocked</t>
-        </is>
-      </c>
-      <c r="B19" s="88" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="107" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ●  Not Started</t>
-        </is>
-      </c>
-      <c r="B20" s="88" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -10135,2396 +9204,272 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="000EA5E9"/>
+    <tabColor rgb="006B7280"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Release Dashboard — All Products 2026</t>
+          <t>How To Use This Tracker</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>At-a-glance: latest release, total count, and next planned for every product</t>
+          <t>Quick guide for all stakeholders</t>
         </is>
       </c>
       <c r="B2" s="4" t="n"/>
       <c r="C2" s="4" t="n"/>
       <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="58" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Sheet</t>
         </is>
       </c>
       <c r="B3" s="58" t="inlineStr">
         <is>
-          <t>Latest Version</t>
+          <t>Purpose</t>
         </is>
       </c>
       <c r="C3" s="58" t="inlineStr">
         <is>
-          <t>Latest Release</t>
+          <t>Update Frequency</t>
         </is>
       </c>
       <c r="D3" s="58" t="inlineStr">
         <is>
-          <t>Release Date</t>
-        </is>
-      </c>
-      <c r="E3" s="58" t="inlineStr">
-        <is>
-          <t>Total Releases</t>
-        </is>
-      </c>
-      <c r="F3" s="58" t="inlineStr">
-        <is>
-          <t>Hotfixes</t>
-        </is>
-      </c>
-      <c r="G3" s="58" t="inlineStr">
-        <is>
-          <t>Next Planned</t>
-        </is>
-      </c>
-      <c r="H3" s="58" t="inlineStr">
-        <is>
-          <t>Next Version</t>
-        </is>
-      </c>
-      <c r="I3" s="58" t="inlineStr">
-        <is>
-          <t>Target Date</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="59" t="inlineStr">
-        <is>
-          <t>📏  Versioning Standard: vMAJOR.MINOR.PATCH  •  Types: MVP | Major | Minor | Hotfix | Patch | Sprint  •  Quarterly releases + hotfixes as needed</t>
-        </is>
-      </c>
-      <c r="B4" s="60" t="n"/>
-      <c r="C4" s="60" t="n"/>
-      <c r="D4" s="60" t="n"/>
-      <c r="E4" s="60" t="n"/>
-      <c r="F4" s="60" t="n"/>
-      <c r="G4" s="60" t="n"/>
-      <c r="H4" s="60" t="n"/>
-      <c r="I4" s="60" t="n"/>
-    </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="49" t="inlineStr">
-        <is>
-          <t>AG ONE</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>v1.0.2</t>
+          <t>Who Updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Team Overview</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>See all 7 internal teams, current sprint, status at a glance</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Every sprint</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Resource Allocation</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Internal + external assignments per member, shared &amp; outsource flags</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>AG ONE Hotfix 2</t>
+          <t>When team changes</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>08 Apr 2026</t>
-        </is>
-      </c>
-      <c r="E5" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="F5" s="62" t="n">
-        <v>2</v>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>AG ONE Q2 Enhancement</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>v1.1.0</t>
-        </is>
-      </c>
-      <c r="I5" s="9" t="inlineStr">
-        <is>
-          <t>May 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="51" t="inlineStr">
-        <is>
-          <t>OneWork</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>v1.0.0</t>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Project Roadmap</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Track project start/end, achievements, next targets, alignment</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>OneWork MVP</t>
+          <t>Every sprint</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>29 Mar 2026</t>
-        </is>
-      </c>
-      <c r="E6" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="13" t="inlineStr">
-        <is>
-          <t>OneWork Q2 Enhancement</t>
-        </is>
-      </c>
-      <c r="H6" s="13" t="inlineStr">
-        <is>
-          <t>v1.1.0</t>
-        </is>
-      </c>
-      <c r="I6" s="13" t="inlineStr">
-        <is>
-          <t>Jun 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="52" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>v1.0.0</t>
+          <t>Tech Leads</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Sprint Tracker</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Detailed sprint goals, outcomes, tech lead feedback, blockers</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Learn MVP</t>
+          <t>Every sprint</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>29 Mar 2026</t>
-        </is>
-      </c>
-      <c r="E7" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>Learn Analytics</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr">
-        <is>
-          <t>v1.1.0</t>
-        </is>
-      </c>
-      <c r="I7" s="9" t="inlineStr">
-        <is>
-          <t>Jun 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="53" t="inlineStr">
-        <is>
-          <t>Safe</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>v1.0.0</t>
+          <t>Tech Leads</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Member Performance</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Individual progress, ratings, achievements</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>Safe MVP</t>
+          <t>Every sprint</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>29 Mar 2026</t>
-        </is>
-      </c>
-      <c r="E8" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="13" t="inlineStr">
-        <is>
-          <t>Safe Regulatory Auto</t>
-        </is>
-      </c>
-      <c r="H8" s="13" t="inlineStr">
-        <is>
-          <t>v1.1.0</t>
-        </is>
-      </c>
-      <c r="I8" s="13" t="inlineStr">
-        <is>
-          <t>Jun 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="54" t="inlineStr">
-        <is>
-          <t>OneHire</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Tech Leads</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>2026 Targets</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Quarterly milestones and year-end goals per team</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Quarterly</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>OneHire Alpha</t>
-        </is>
-      </c>
-      <c r="H9" s="9" t="inlineStr">
-        <is>
-          <t>v0.1.0</t>
-        </is>
-      </c>
-      <c r="I9" s="9" t="inlineStr">
-        <is>
-          <t>May 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="55" t="inlineStr">
-        <is>
-          <t>Spot</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>External Projects</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Track resources on external / outsource / partner projects</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>When assignments change</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>Spot Alpha</t>
-        </is>
-      </c>
-      <c r="H10" s="13" t="inlineStr">
-        <is>
-          <t>v0.1.0</t>
-        </is>
-      </c>
-      <c r="I10" s="13" t="inlineStr">
-        <is>
-          <t>May 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="56" t="inlineStr">
-        <is>
-          <t>Pulse</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>Pulse Alpha</t>
-        </is>
-      </c>
-      <c r="H11" s="9" t="inlineStr">
-        <is>
-          <t>v0.1.0</t>
-        </is>
-      </c>
-      <c r="I11" s="9" t="inlineStr">
-        <is>
-          <t>May 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="59" t="inlineStr">
+        <is>
+          <t>STATUS LEGEND</t>
+        </is>
+      </c>
+    </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>TOTAL ACROSS ALL PRODUCTS</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="F13" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="G13" s="64" t="inlineStr">
-        <is>
-          <t>19 releases planned</t>
-        </is>
-      </c>
-      <c r="H13" s="65" t="n"/>
-      <c r="I13" s="65" t="n"/>
+      <c r="A13" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ●  ✅ Completed</t>
+        </is>
+      </c>
+      <c r="B13" s="61" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ●  ▶ In Progress / On Track</t>
+        </is>
+      </c>
+      <c r="B14" s="61" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ●  At Risk</t>
+        </is>
+      </c>
+      <c r="B15" s="61" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ●  Blocked</t>
+        </is>
+      </c>
+      <c r="B16" s="61" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ●  Not Started</t>
+        </is>
+      </c>
+      <c r="B17" s="61" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="A13:D13"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="000284C7"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I68"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="55" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Release History — All Products 2026</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Every release grouped by product: Released ✅ + Upcoming 📋  •  Scroll down for each team</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="66" t="inlineStr">
-        <is>
-          <t>AG ONE  —  Released: 3  •  Hotfixes: 2  •  Planned: 3  •  Latest: v1.0.2  •  Next: v1.1.0</t>
-        </is>
-      </c>
-      <c r="B3" s="67" t="n"/>
-      <c r="C3" s="67" t="n"/>
-      <c r="D3" s="67" t="n"/>
-      <c r="E3" s="67" t="n"/>
-      <c r="F3" s="67" t="n"/>
-      <c r="G3" s="67" t="n"/>
-      <c r="H3" s="67" t="n"/>
-      <c r="I3" s="67" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="68" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B4" s="68" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="C4" s="68" t="inlineStr">
-        <is>
-          <t>Version</t>
-        </is>
-      </c>
-      <c r="D4" s="68" t="inlineStr">
-        <is>
-          <t>Release Name</t>
-        </is>
-      </c>
-      <c r="E4" s="68" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="F4" s="68" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="G4" s="68" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="H4" s="68" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="I4" s="68" t="inlineStr">
-        <is>
-          <t>Highlights / What's Included</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>AG ONE</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>v1.0.0</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>AG ONE MVP</t>
-        </is>
-      </c>
-      <c r="E5" s="69" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>29 Mar 2026</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 6</t>
-        </is>
-      </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>✅ Released</t>
-        </is>
-      </c>
-      <c r="I5" s="10" t="inlineStr">
-        <is>
-          <t>Full IAM platform: Users, Roles, Tenants, SSO, Permissions, Audit, Assign Access</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>AG ONE</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="inlineStr">
-        <is>
-          <t>v1.0.1</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>AG ONE Hotfix 1</t>
-        </is>
-      </c>
-      <c r="E6" s="70" t="inlineStr">
-        <is>
-          <t>Hotfix</t>
-        </is>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
-        <is>
-          <t>02 Apr 2026</t>
-        </is>
-      </c>
-      <c r="G6" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 7</t>
-        </is>
-      </c>
-      <c r="H6" s="11" t="inlineStr">
-        <is>
-          <t>✅ Released</t>
-        </is>
-      </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>SSO token refresh loop fix, role sync cache invalidation, tenant switching fix</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>AG ONE</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>v1.0.2</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>AG ONE Hotfix 2</t>
-        </is>
-      </c>
-      <c r="E7" s="70" t="inlineStr">
-        <is>
-          <t>Hotfix</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>08 Apr 2026</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 7</t>
-        </is>
-      </c>
-      <c r="H7" s="11" t="inlineStr">
-        <is>
-          <t>✅ Released</t>
-        </is>
-      </c>
-      <c r="I7" s="10" t="inlineStr">
-        <is>
-          <t>Audit log pagination, API key duplicate name validation, timezone fix</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>AG ONE</t>
-        </is>
-      </c>
-      <c r="C8" s="13" t="inlineStr">
-        <is>
-          <t>v1.1.0</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>AG ONE Q2 Enhancement</t>
-        </is>
-      </c>
-      <c r="E8" s="71" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="F8" s="13" t="inlineStr">
-        <is>
-          <t>May 2026</t>
-        </is>
-      </c>
-      <c r="G8" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 9–10</t>
-        </is>
-      </c>
-      <c r="H8" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I8" s="14" t="inlineStr">
-        <is>
-          <t>Advanced user analytics, bulk role operations, enhanced audit dashboard</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>AG ONE</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>v1.2.0</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>AG ONE Multi-Product Admin</t>
-        </is>
-      </c>
-      <c r="E9" s="71" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>Jul 2026</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 13–14</t>
-        </is>
-      </c>
-      <c r="H9" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I9" s="10" t="inlineStr">
-        <is>
-          <t>Multi-product admin console, cross-product role mapping, API marketplace v1</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>AG ONE</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>v2.0.0</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>AG ONE Enterprise</t>
-        </is>
-      </c>
-      <c r="E10" s="71" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
-        <is>
-          <t>Oct 2026</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 20–22</t>
-        </is>
-      </c>
-      <c r="H10" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I10" s="14" t="inlineStr">
-        <is>
-          <t>Enterprise SSO (SAML+OIDC), advanced RBAC, white-label branding, scale</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr"/>
-      <c r="B11" s="72" t="inlineStr">
-        <is>
-          <t>AG ONE</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="9" t="n"/>
-      <c r="F11" s="9" t="n"/>
-      <c r="G11" s="9" t="n"/>
-      <c r="H11" s="9" t="n"/>
-      <c r="I11" s="10" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="13" t="inlineStr"/>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>AG ONE</t>
-        </is>
-      </c>
-      <c r="C12" s="13" t="n"/>
-      <c r="D12" s="14" t="n"/>
-      <c r="E12" s="13" t="n"/>
-      <c r="F12" s="13" t="n"/>
-      <c r="G12" s="13" t="n"/>
-      <c r="H12" s="13" t="n"/>
-      <c r="I12" s="14" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr"/>
-      <c r="B13" s="72" t="inlineStr">
-        <is>
-          <t>AG ONE</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="9" t="n"/>
-      <c r="F13" s="9" t="n"/>
-      <c r="G13" s="9" t="n"/>
-      <c r="H13" s="9" t="n"/>
-      <c r="I13" s="10" t="n"/>
-    </row>
-    <row r="14"/>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="73" t="inlineStr">
-        <is>
-          <t>OneWork  —  Released: 1  •  Hotfixes: 0  •  Planned: 3  •  Latest: v1.0.0  •  Next: v1.1.0</t>
-        </is>
-      </c>
-      <c r="B15" s="74" t="n"/>
-      <c r="C15" s="74" t="n"/>
-      <c r="D15" s="74" t="n"/>
-      <c r="E15" s="74" t="n"/>
-      <c r="F15" s="74" t="n"/>
-      <c r="G15" s="74" t="n"/>
-      <c r="H15" s="74" t="n"/>
-      <c r="I15" s="74" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="68" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B16" s="68" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="C16" s="68" t="inlineStr">
-        <is>
-          <t>Version</t>
-        </is>
-      </c>
-      <c r="D16" s="68" t="inlineStr">
-        <is>
-          <t>Release Name</t>
-        </is>
-      </c>
-      <c r="E16" s="68" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="F16" s="68" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="G16" s="68" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="H16" s="68" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="I16" s="68" t="inlineStr">
-        <is>
-          <t>Highlights / What's Included</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>OneWork</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>v1.0.0</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>OneWork MVP</t>
-        </is>
-      </c>
-      <c r="E17" s="69" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>29 Mar 2026</t>
-        </is>
-      </c>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 6</t>
-        </is>
-      </c>
-      <c r="H17" s="11" t="inlineStr">
-        <is>
-          <t>✅ Released</t>
-        </is>
-      </c>
-      <c r="I17" s="10" t="inlineStr">
-        <is>
-          <t>Employee mgmt, workflows, task mgmt, dashboards, reporting</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="13" t="n">
-        <v>11</v>
-      </c>
-      <c r="B18" s="13" t="inlineStr">
-        <is>
-          <t>OneWork</t>
-        </is>
-      </c>
-      <c r="C18" s="13" t="inlineStr">
-        <is>
-          <t>v1.1.0</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>OneWork Q2 Enhancement</t>
-        </is>
-      </c>
-      <c r="E18" s="71" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
-        <is>
-          <t>Jun 2026</t>
-        </is>
-      </c>
-      <c r="G18" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 11–12</t>
-        </is>
-      </c>
-      <c r="H18" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I18" s="14" t="inlineStr">
-        <is>
-          <t>Advanced workflow templates, email notifications, calendar integration</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>OneWork</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>v1.2.0</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>OneWork Reporting v2</t>
-        </is>
-      </c>
-      <c r="E19" s="71" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="F19" s="9" t="inlineStr">
-        <is>
-          <t>Aug 2026</t>
-        </is>
-      </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 15–16</t>
-        </is>
-      </c>
-      <c r="H19" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I19" s="10" t="inlineStr">
-        <is>
-          <t>Reporting v2 with charts, mobile-responsive, third-party integrations</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="13" t="n">
-        <v>13</v>
-      </c>
-      <c r="B20" s="13" t="inlineStr">
-        <is>
-          <t>OneWork</t>
-        </is>
-      </c>
-      <c r="C20" s="13" t="inlineStr">
-        <is>
-          <t>v2.0.0</t>
-        </is>
-      </c>
-      <c r="D20" s="14" t="inlineStr">
-        <is>
-          <t>OneWork Enterprise</t>
-        </is>
-      </c>
-      <c r="E20" s="71" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="inlineStr">
-        <is>
-          <t>Nov 2026</t>
-        </is>
-      </c>
-      <c r="G20" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 21–23</t>
-        </is>
-      </c>
-      <c r="H20" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I20" s="14" t="inlineStr">
-        <is>
-          <t>AI-powered insights, advanced automation, enterprise scale</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr"/>
-      <c r="B21" s="72" t="inlineStr">
-        <is>
-          <t>OneWork</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="n"/>
-      <c r="D21" s="10" t="n"/>
-      <c r="E21" s="9" t="n"/>
-      <c r="F21" s="9" t="n"/>
-      <c r="G21" s="9" t="n"/>
-      <c r="H21" s="9" t="n"/>
-      <c r="I21" s="10" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="13" t="inlineStr"/>
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>OneWork</t>
-        </is>
-      </c>
-      <c r="C22" s="13" t="n"/>
-      <c r="D22" s="14" t="n"/>
-      <c r="E22" s="13" t="n"/>
-      <c r="F22" s="13" t="n"/>
-      <c r="G22" s="13" t="n"/>
-      <c r="H22" s="13" t="n"/>
-      <c r="I22" s="14" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr"/>
-      <c r="B23" s="72" t="inlineStr">
-        <is>
-          <t>OneWork</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="n"/>
-      <c r="D23" s="10" t="n"/>
-      <c r="E23" s="9" t="n"/>
-      <c r="F23" s="9" t="n"/>
-      <c r="G23" s="9" t="n"/>
-      <c r="H23" s="9" t="n"/>
-      <c r="I23" s="10" t="n"/>
-    </row>
-    <row r="24"/>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="75" t="inlineStr">
-        <is>
-          <t>Learn  —  Released: 1  •  Hotfixes: 0  •  Planned: 3  •  Latest: v1.0.0  •  Next: v1.1.0</t>
-        </is>
-      </c>
-      <c r="B25" s="76" t="n"/>
-      <c r="C25" s="76" t="n"/>
-      <c r="D25" s="76" t="n"/>
-      <c r="E25" s="76" t="n"/>
-      <c r="F25" s="76" t="n"/>
-      <c r="G25" s="76" t="n"/>
-      <c r="H25" s="76" t="n"/>
-      <c r="I25" s="76" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="68" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B26" s="68" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="C26" s="68" t="inlineStr">
-        <is>
-          <t>Version</t>
-        </is>
-      </c>
-      <c r="D26" s="68" t="inlineStr">
-        <is>
-          <t>Release Name</t>
-        </is>
-      </c>
-      <c r="E26" s="68" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="F26" s="68" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="G26" s="68" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="H26" s="68" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="I26" s="68" t="inlineStr">
-        <is>
-          <t>Highlights / What's Included</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="9" t="n">
-        <v>17</v>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>v1.0.0</t>
-        </is>
-      </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>Learn MVP</t>
-        </is>
-      </c>
-      <c r="E27" s="69" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="F27" s="9" t="inlineStr">
-        <is>
-          <t>29 Mar 2026</t>
-        </is>
-      </c>
-      <c r="G27" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 6</t>
-        </is>
-      </c>
-      <c r="H27" s="11" t="inlineStr">
-        <is>
-          <t>✅ Released</t>
-        </is>
-      </c>
-      <c r="I27" s="10" t="inlineStr">
-        <is>
-          <t>Courses, learning paths, assessments, certifications, progress tracking</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="13" t="n">
-        <v>18</v>
-      </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="C28" s="13" t="inlineStr">
-        <is>
-          <t>v1.1.0</t>
-        </is>
-      </c>
-      <c r="D28" s="14" t="inlineStr">
-        <is>
-          <t>Learn Analytics</t>
-        </is>
-      </c>
-      <c r="E28" s="71" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
-        <is>
-          <t>Jun 2026</t>
-        </is>
-      </c>
-      <c r="G28" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 11–12</t>
-        </is>
-      </c>
-      <c r="H28" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I28" s="14" t="inlineStr">
-        <is>
-          <t>Advanced analytics dashboard, learner recommendations, completion reports</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="9" t="n">
-        <v>19</v>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>v1.2.0</t>
-        </is>
-      </c>
-      <c r="D29" s="10" t="inlineStr">
-        <is>
-          <t>Learn Marketplace</t>
-        </is>
-      </c>
-      <c r="E29" s="71" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="F29" s="9" t="inlineStr">
-        <is>
-          <t>Aug 2026</t>
-        </is>
-      </c>
-      <c r="G29" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 15–16</t>
-        </is>
-      </c>
-      <c r="H29" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I29" s="10" t="inlineStr">
-        <is>
-          <t>Content marketplace, SCORM support, mobile-responsive learning</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="13" t="n">
-        <v>20</v>
-      </c>
-      <c r="B30" s="13" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="C30" s="13" t="inlineStr">
-        <is>
-          <t>v2.0.0</t>
-        </is>
-      </c>
-      <c r="D30" s="14" t="inlineStr">
-        <is>
-          <t>Learn Enterprise</t>
-        </is>
-      </c>
-      <c r="E30" s="71" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="inlineStr">
-        <is>
-          <t>Nov 2026</t>
-        </is>
-      </c>
-      <c r="G30" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 21–23</t>
-        </is>
-      </c>
-      <c r="H30" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I30" s="14" t="inlineStr">
-        <is>
-          <t>AI recommendations, adaptive learning, full mobile app</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="inlineStr"/>
-      <c r="B31" s="72" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="n"/>
-      <c r="D31" s="10" t="n"/>
-      <c r="E31" s="9" t="n"/>
-      <c r="F31" s="9" t="n"/>
-      <c r="G31" s="9" t="n"/>
-      <c r="H31" s="9" t="n"/>
-      <c r="I31" s="10" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="13" t="inlineStr"/>
-      <c r="B32" s="18" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="C32" s="13" t="n"/>
-      <c r="D32" s="14" t="n"/>
-      <c r="E32" s="13" t="n"/>
-      <c r="F32" s="13" t="n"/>
-      <c r="G32" s="13" t="n"/>
-      <c r="H32" s="13" t="n"/>
-      <c r="I32" s="14" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="9" t="inlineStr"/>
-      <c r="B33" s="72" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="n"/>
-      <c r="D33" s="10" t="n"/>
-      <c r="E33" s="9" t="n"/>
-      <c r="F33" s="9" t="n"/>
-      <c r="G33" s="9" t="n"/>
-      <c r="H33" s="9" t="n"/>
-      <c r="I33" s="10" t="n"/>
-    </row>
-    <row r="34"/>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="77" t="inlineStr">
-        <is>
-          <t>Safe  —  Released: 1  •  Hotfixes: 0  •  Planned: 3  •  Latest: v1.0.0  •  Next: v1.1.0</t>
-        </is>
-      </c>
-      <c r="B35" s="78" t="n"/>
-      <c r="C35" s="78" t="n"/>
-      <c r="D35" s="78" t="n"/>
-      <c r="E35" s="78" t="n"/>
-      <c r="F35" s="78" t="n"/>
-      <c r="G35" s="78" t="n"/>
-      <c r="H35" s="78" t="n"/>
-      <c r="I35" s="78" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="68" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B36" s="68" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="C36" s="68" t="inlineStr">
-        <is>
-          <t>Version</t>
-        </is>
-      </c>
-      <c r="D36" s="68" t="inlineStr">
-        <is>
-          <t>Release Name</t>
-        </is>
-      </c>
-      <c r="E36" s="68" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="F36" s="68" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="G36" s="68" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="H36" s="68" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="I36" s="68" t="inlineStr">
-        <is>
-          <t>Highlights / What's Included</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="9" t="n">
-        <v>24</v>
-      </c>
-      <c r="B37" s="9" t="inlineStr">
-        <is>
-          <t>Safe</t>
-        </is>
-      </c>
-      <c r="C37" s="9" t="inlineStr">
-        <is>
-          <t>v1.0.0</t>
-        </is>
-      </c>
-      <c r="D37" s="10" t="inlineStr">
-        <is>
-          <t>Safe MVP</t>
-        </is>
-      </c>
-      <c r="E37" s="69" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="inlineStr">
-        <is>
-          <t>29 Mar 2026</t>
-        </is>
-      </c>
-      <c r="G37" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 6</t>
-        </is>
-      </c>
-      <c r="H37" s="11" t="inlineStr">
-        <is>
-          <t>✅ Released</t>
-        </is>
-      </c>
-      <c r="I37" s="10" t="inlineStr">
-        <is>
-          <t>Policies, compliance tracking, audit workflows, risk matrix, dashboards</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="13" t="n">
-        <v>25</v>
-      </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>Safe</t>
-        </is>
-      </c>
-      <c r="C38" s="13" t="inlineStr">
-        <is>
-          <t>v1.1.0</t>
-        </is>
-      </c>
-      <c r="D38" s="14" t="inlineStr">
-        <is>
-          <t>Safe Regulatory Auto</t>
-        </is>
-      </c>
-      <c r="E38" s="71" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="F38" s="13" t="inlineStr">
-        <is>
-          <t>Jun 2026</t>
-        </is>
-      </c>
-      <c r="G38" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 11–12</t>
-        </is>
-      </c>
-      <c r="H38" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I38" s="14" t="inlineStr">
-        <is>
-          <t>Regulatory update automation, scheduled compliance checks, advanced reporting</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="B39" s="9" t="inlineStr">
-        <is>
-          <t>Safe</t>
-        </is>
-      </c>
-      <c r="C39" s="9" t="inlineStr">
-        <is>
-          <t>v1.2.0</t>
-        </is>
-      </c>
-      <c r="D39" s="10" t="inlineStr">
-        <is>
-          <t>Safe Integrations</t>
-        </is>
-      </c>
-      <c r="E39" s="71" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-      <c r="G39" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 17–18</t>
-        </is>
-      </c>
-      <c r="H39" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I39" s="10" t="inlineStr">
-        <is>
-          <t>Third-party GRC integrations, automated alerts, evidence collection</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="13" t="n">
-        <v>27</v>
-      </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>Safe</t>
-        </is>
-      </c>
-      <c r="C40" s="13" t="inlineStr">
-        <is>
-          <t>v2.0.0</t>
-        </is>
-      </c>
-      <c r="D40" s="14" t="inlineStr">
-        <is>
-          <t>Safe Enterprise</t>
-        </is>
-      </c>
-      <c r="E40" s="71" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="F40" s="13" t="inlineStr">
-        <is>
-          <t>Dec 2026</t>
-        </is>
-      </c>
-      <c r="G40" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 24–26</t>
-        </is>
-      </c>
-      <c r="H40" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I40" s="14" t="inlineStr">
-        <is>
-          <t>Enterprise compliance suite with AI-driven risk predictions</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="9" t="inlineStr"/>
-      <c r="B41" s="72" t="inlineStr">
-        <is>
-          <t>Safe</t>
-        </is>
-      </c>
-      <c r="C41" s="9" t="n"/>
-      <c r="D41" s="10" t="n"/>
-      <c r="E41" s="9" t="n"/>
-      <c r="F41" s="9" t="n"/>
-      <c r="G41" s="9" t="n"/>
-      <c r="H41" s="9" t="n"/>
-      <c r="I41" s="10" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="13" t="inlineStr"/>
-      <c r="B42" s="18" t="inlineStr">
-        <is>
-          <t>Safe</t>
-        </is>
-      </c>
-      <c r="C42" s="13" t="n"/>
-      <c r="D42" s="14" t="n"/>
-      <c r="E42" s="13" t="n"/>
-      <c r="F42" s="13" t="n"/>
-      <c r="G42" s="13" t="n"/>
-      <c r="H42" s="13" t="n"/>
-      <c r="I42" s="14" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="9" t="inlineStr"/>
-      <c r="B43" s="72" t="inlineStr">
-        <is>
-          <t>Safe</t>
-        </is>
-      </c>
-      <c r="C43" s="9" t="n"/>
-      <c r="D43" s="10" t="n"/>
-      <c r="E43" s="9" t="n"/>
-      <c r="F43" s="9" t="n"/>
-      <c r="G43" s="9" t="n"/>
-      <c r="H43" s="9" t="n"/>
-      <c r="I43" s="10" t="n"/>
-    </row>
-    <row r="44"/>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="79" t="inlineStr">
-        <is>
-          <t>OneHire  —  Released: 0  •  Hotfixes: 0  •  Planned: 3  •  Latest: —  •  Next: v0.1.0</t>
-        </is>
-      </c>
-      <c r="B45" s="80" t="n"/>
-      <c r="C45" s="80" t="n"/>
-      <c r="D45" s="80" t="n"/>
-      <c r="E45" s="80" t="n"/>
-      <c r="F45" s="80" t="n"/>
-      <c r="G45" s="80" t="n"/>
-      <c r="H45" s="80" t="n"/>
-      <c r="I45" s="80" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="68" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B46" s="68" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="C46" s="68" t="inlineStr">
-        <is>
-          <t>Version</t>
-        </is>
-      </c>
-      <c r="D46" s="68" t="inlineStr">
-        <is>
-          <t>Release Name</t>
-        </is>
-      </c>
-      <c r="E46" s="68" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="F46" s="68" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="G46" s="68" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="H46" s="68" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="I46" s="68" t="inlineStr">
-        <is>
-          <t>Highlights / What's Included</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="9" t="n">
-        <v>31</v>
-      </c>
-      <c r="B47" s="9" t="inlineStr">
-        <is>
-          <t>OneHire</t>
-        </is>
-      </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>v0.1.0</t>
-        </is>
-      </c>
-      <c r="D47" s="10" t="inlineStr">
-        <is>
-          <t>OneHire Alpha</t>
-        </is>
-      </c>
-      <c r="E47" s="81" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="inlineStr">
-        <is>
-          <t>May 2026</t>
-        </is>
-      </c>
-      <c r="G47" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 9–10</t>
-        </is>
-      </c>
-      <c r="H47" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I47" s="10" t="inlineStr">
-        <is>
-          <t>Core job posting and applicant tracking features</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="13" t="n">
-        <v>32</v>
-      </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>OneHire</t>
-        </is>
-      </c>
-      <c r="C48" s="13" t="inlineStr">
-        <is>
-          <t>v0.5.0</t>
-        </is>
-      </c>
-      <c r="D48" s="14" t="inlineStr">
-        <is>
-          <t>OneHire Beta</t>
-        </is>
-      </c>
-      <c r="E48" s="81" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="F48" s="13" t="inlineStr">
-        <is>
-          <t>Jun 2026</t>
-        </is>
-      </c>
-      <c r="G48" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 11–12</t>
-        </is>
-      </c>
-      <c r="H48" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I48" s="14" t="inlineStr">
-        <is>
-          <t>Interview scheduling, candidate pipeline, basic reporting</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="30" customHeight="1">
-      <c r="A49" s="9" t="n">
-        <v>33</v>
-      </c>
-      <c r="B49" s="9" t="inlineStr">
-        <is>
-          <t>OneHire</t>
-        </is>
-      </c>
-      <c r="C49" s="9" t="inlineStr">
-        <is>
-          <t>v1.0.0</t>
-        </is>
-      </c>
-      <c r="D49" s="10" t="inlineStr">
-        <is>
-          <t>OneHire MVP</t>
-        </is>
-      </c>
-      <c r="E49" s="69" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="inlineStr">
-        <is>
-          <t>Jul 2026</t>
-        </is>
-      </c>
-      <c r="G49" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 13–14</t>
-        </is>
-      </c>
-      <c r="H49" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I49" s="10" t="inlineStr">
-        <is>
-          <t>Full recruitment portal with applicant tracking and analytics</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="13" t="inlineStr"/>
-      <c r="B50" s="18" t="inlineStr">
-        <is>
-          <t>OneHire</t>
-        </is>
-      </c>
-      <c r="C50" s="13" t="n"/>
-      <c r="D50" s="14" t="n"/>
-      <c r="E50" s="13" t="n"/>
-      <c r="F50" s="13" t="n"/>
-      <c r="G50" s="13" t="n"/>
-      <c r="H50" s="13" t="n"/>
-      <c r="I50" s="14" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="9" t="inlineStr"/>
-      <c r="B51" s="72" t="inlineStr">
-        <is>
-          <t>OneHire</t>
-        </is>
-      </c>
-      <c r="C51" s="9" t="n"/>
-      <c r="D51" s="10" t="n"/>
-      <c r="E51" s="9" t="n"/>
-      <c r="F51" s="9" t="n"/>
-      <c r="G51" s="9" t="n"/>
-      <c r="H51" s="9" t="n"/>
-      <c r="I51" s="10" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="13" t="inlineStr"/>
-      <c r="B52" s="18" t="inlineStr">
-        <is>
-          <t>OneHire</t>
-        </is>
-      </c>
-      <c r="C52" s="13" t="n"/>
-      <c r="D52" s="14" t="n"/>
-      <c r="E52" s="13" t="n"/>
-      <c r="F52" s="13" t="n"/>
-      <c r="G52" s="13" t="n"/>
-      <c r="H52" s="13" t="n"/>
-      <c r="I52" s="14" t="n"/>
-    </row>
-    <row r="53"/>
-    <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="82" t="inlineStr">
-        <is>
-          <t>Spot  —  Released: 0  •  Hotfixes: 0  •  Planned: 2  •  Latest: —  •  Next: v0.1.0</t>
-        </is>
-      </c>
-      <c r="B54" s="83" t="n"/>
-      <c r="C54" s="83" t="n"/>
-      <c r="D54" s="83" t="n"/>
-      <c r="E54" s="83" t="n"/>
-      <c r="F54" s="83" t="n"/>
-      <c r="G54" s="83" t="n"/>
-      <c r="H54" s="83" t="n"/>
-      <c r="I54" s="83" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="68" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B55" s="68" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="C55" s="68" t="inlineStr">
-        <is>
-          <t>Version</t>
-        </is>
-      </c>
-      <c r="D55" s="68" t="inlineStr">
-        <is>
-          <t>Release Name</t>
-        </is>
-      </c>
-      <c r="E55" s="68" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="F55" s="68" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="G55" s="68" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="H55" s="68" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="I55" s="68" t="inlineStr">
-        <is>
-          <t>Highlights / What's Included</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="30" customHeight="1">
-      <c r="A56" s="13" t="n">
-        <v>37</v>
-      </c>
-      <c r="B56" s="13" t="inlineStr">
-        <is>
-          <t>Spot</t>
-        </is>
-      </c>
-      <c r="C56" s="13" t="inlineStr">
-        <is>
-          <t>v0.1.0</t>
-        </is>
-      </c>
-      <c r="D56" s="14" t="inlineStr">
-        <is>
-          <t>Spot Alpha</t>
-        </is>
-      </c>
-      <c r="E56" s="81" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="F56" s="13" t="inlineStr">
-        <is>
-          <t>May 2026</t>
-        </is>
-      </c>
-      <c r="G56" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 9–10</t>
-        </is>
-      </c>
-      <c r="H56" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I56" s="14" t="inlineStr">
-        <is>
-          <t>Core city module, location management</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="9" t="n">
-        <v>38</v>
-      </c>
-      <c r="B57" s="9" t="inlineStr">
-        <is>
-          <t>Spot</t>
-        </is>
-      </c>
-      <c r="C57" s="9" t="inlineStr">
-        <is>
-          <t>v1.0.0</t>
-        </is>
-      </c>
-      <c r="D57" s="10" t="inlineStr">
-        <is>
-          <t>Spot MVP</t>
-        </is>
-      </c>
-      <c r="E57" s="69" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-      <c r="G57" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 17–18</t>
-        </is>
-      </c>
-      <c r="H57" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I57" s="10" t="inlineStr">
-        <is>
-          <t>City management, geolocation features, admin dashboard</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="13" t="inlineStr"/>
-      <c r="B58" s="18" t="inlineStr">
-        <is>
-          <t>Spot</t>
-        </is>
-      </c>
-      <c r="C58" s="13" t="n"/>
-      <c r="D58" s="14" t="n"/>
-      <c r="E58" s="13" t="n"/>
-      <c r="F58" s="13" t="n"/>
-      <c r="G58" s="13" t="n"/>
-      <c r="H58" s="13" t="n"/>
-      <c r="I58" s="14" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="9" t="inlineStr"/>
-      <c r="B59" s="72" t="inlineStr">
-        <is>
-          <t>Spot</t>
-        </is>
-      </c>
-      <c r="C59" s="9" t="n"/>
-      <c r="D59" s="10" t="n"/>
-      <c r="E59" s="9" t="n"/>
-      <c r="F59" s="9" t="n"/>
-      <c r="G59" s="9" t="n"/>
-      <c r="H59" s="9" t="n"/>
-      <c r="I59" s="10" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="13" t="inlineStr"/>
-      <c r="B60" s="18" t="inlineStr">
-        <is>
-          <t>Spot</t>
-        </is>
-      </c>
-      <c r="C60" s="13" t="n"/>
-      <c r="D60" s="14" t="n"/>
-      <c r="E60" s="13" t="n"/>
-      <c r="F60" s="13" t="n"/>
-      <c r="G60" s="13" t="n"/>
-      <c r="H60" s="13" t="n"/>
-      <c r="I60" s="14" t="n"/>
-    </row>
-    <row r="61"/>
-    <row r="62" ht="30" customHeight="1">
-      <c r="A62" s="84" t="inlineStr">
-        <is>
-          <t>Pulse  —  Released: 0  •  Hotfixes: 0  •  Planned: 2  •  Latest: —  •  Next: v0.1.0</t>
-        </is>
-      </c>
-      <c r="B62" s="85" t="n"/>
-      <c r="C62" s="85" t="n"/>
-      <c r="D62" s="85" t="n"/>
-      <c r="E62" s="85" t="n"/>
-      <c r="F62" s="85" t="n"/>
-      <c r="G62" s="85" t="n"/>
-      <c r="H62" s="85" t="n"/>
-      <c r="I62" s="85" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="68" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B63" s="68" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="C63" s="68" t="inlineStr">
-        <is>
-          <t>Version</t>
-        </is>
-      </c>
-      <c r="D63" s="68" t="inlineStr">
-        <is>
-          <t>Release Name</t>
-        </is>
-      </c>
-      <c r="E63" s="68" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="F63" s="68" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="G63" s="68" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="H63" s="68" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="I63" s="68" t="inlineStr">
-        <is>
-          <t>Highlights / What's Included</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="30" customHeight="1">
-      <c r="A64" s="13" t="n">
-        <v>42</v>
-      </c>
-      <c r="B64" s="13" t="inlineStr">
-        <is>
-          <t>Pulse</t>
-        </is>
-      </c>
-      <c r="C64" s="13" t="inlineStr">
-        <is>
-          <t>v0.1.0</t>
-        </is>
-      </c>
-      <c r="D64" s="14" t="inlineStr">
-        <is>
-          <t>Pulse Alpha</t>
-        </is>
-      </c>
-      <c r="E64" s="81" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="F64" s="13" t="inlineStr">
-        <is>
-          <t>May 2026</t>
-        </is>
-      </c>
-      <c r="G64" s="13" t="inlineStr">
-        <is>
-          <t>Sprint 9–10</t>
-        </is>
-      </c>
-      <c r="H64" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I64" s="14" t="inlineStr">
-        <is>
-          <t>Survey builder, basic distribution</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="30" customHeight="1">
-      <c r="A65" s="9" t="n">
-        <v>43</v>
-      </c>
-      <c r="B65" s="9" t="inlineStr">
-        <is>
-          <t>Pulse</t>
-        </is>
-      </c>
-      <c r="C65" s="9" t="inlineStr">
-        <is>
-          <t>v1.0.0</t>
-        </is>
-      </c>
-      <c r="D65" s="10" t="inlineStr">
-        <is>
-          <t>Pulse MVP</t>
-        </is>
-      </c>
-      <c r="E65" s="69" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="F65" s="9" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-      <c r="G65" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 17–18</t>
-        </is>
-      </c>
-      <c r="H65" s="18" t="inlineStr">
-        <is>
-          <t>📋 Planned</t>
-        </is>
-      </c>
-      <c r="I65" s="10" t="inlineStr">
-        <is>
-          <t>Survey analytics, employee engagement dashboards, benchmarking</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="13" t="inlineStr"/>
-      <c r="B66" s="18" t="inlineStr">
-        <is>
-          <t>Pulse</t>
-        </is>
-      </c>
-      <c r="C66" s="13" t="n"/>
-      <c r="D66" s="14" t="n"/>
-      <c r="E66" s="13" t="n"/>
-      <c r="F66" s="13" t="n"/>
-      <c r="G66" s="13" t="n"/>
-      <c r="H66" s="13" t="n"/>
-      <c r="I66" s="14" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="9" t="inlineStr"/>
-      <c r="B67" s="72" t="inlineStr">
-        <is>
-          <t>Pulse</t>
-        </is>
-      </c>
-      <c r="C67" s="9" t="n"/>
-      <c r="D67" s="10" t="n"/>
-      <c r="E67" s="9" t="n"/>
-      <c r="F67" s="9" t="n"/>
-      <c r="G67" s="9" t="n"/>
-      <c r="H67" s="9" t="n"/>
-      <c r="I67" s="10" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="13" t="inlineStr"/>
-      <c r="B68" s="18" t="inlineStr">
-        <is>
-          <t>Pulse</t>
-        </is>
-      </c>
-      <c r="C68" s="13" t="n"/>
-      <c r="D68" s="14" t="n"/>
-      <c r="E68" s="13" t="n"/>
-      <c r="F68" s="13" t="n"/>
-      <c r="G68" s="13" t="n"/>
-      <c r="H68" s="13" t="n"/>
-      <c r="I68" s="14" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A15:I15"/>
-    <mergeCell ref="A25:I25"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A45:I45"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A35:I35"/>
-    <mergeCell ref="A62:I62"/>
-    <mergeCell ref="A54:I54"/>
+  <mergeCells count="7">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A17:B17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>

</xml_diff>